<commit_message>
still troubleshooting fact_driver_race table
</commit_message>
<xml_diff>
--- a/data/raw/newHistPointAndPrice.xlsx
+++ b/data/raw/newHistPointAndPrice.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F031A4B9-18A7-49AD-930A-50D4B413A350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BC5BF65-EA33-4282-9FED-9F92A4F5ED39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" firstSheet="7" activeTab="16" xr2:uid="{2D04FC15-E09F-4251-B381-E10D89E9EC62}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="864" firstSheet="9" activeTab="11" xr2:uid="{2D04FC15-E09F-4251-B381-E10D89E9EC62}"/>
   </bookViews>
   <sheets>
     <sheet name="2023ConstructorPrice" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="84">
   <si>
     <t>Red Bull Racing</t>
   </si>
@@ -701,9 +701,9 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:W11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -774,7 +774,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="15.75">
+    <row r="2" spans="1:23" ht="15.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -845,7 +845,7 @@
         <v>29.7</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="15.75">
+    <row r="3" spans="1:23" ht="15.4">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -916,7 +916,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="15.75">
+    <row r="4" spans="1:23" ht="15.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -987,7 +987,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="15.75">
+    <row r="5" spans="1:23" ht="15.4">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1058,7 +1058,7 @@
         <v>17.100000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="15.75">
+    <row r="6" spans="1:23" ht="15.4">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1129,7 +1129,7 @@
         <v>14.2</v>
       </c>
     </row>
-    <row r="7" spans="1:23" ht="15.75">
+    <row r="7" spans="1:23" ht="15.4">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -1200,7 +1200,7 @@
         <v>13.4</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="15.75">
+    <row r="8" spans="1:23" ht="15.4">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1271,7 +1271,7 @@
         <v>8.6999999999999993</v>
       </c>
     </row>
-    <row r="9" spans="1:23" ht="15.75">
+    <row r="9" spans="1:23" ht="15.4">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1342,7 +1342,7 @@
         <v>6.6</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="15.75">
+    <row r="10" spans="1:23" ht="15.4">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1413,7 +1413,7 @@
         <v>7.8</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="15.75">
+    <row r="11" spans="1:23" ht="15.4">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1495,9 +1495,9 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:Y26"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25">
@@ -1574,7 +1574,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="15.75">
+    <row r="2" spans="1:25" ht="15.4">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1651,7 +1651,7 @@
         <v>32.299999999999997</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15.75">
+    <row r="3" spans="1:25" ht="15.4">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -1728,7 +1728,7 @@
         <v>27.5</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.75">
+    <row r="4" spans="1:25" ht="15.4">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1805,7 +1805,7 @@
         <v>26.1</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="15.75">
+    <row r="5" spans="1:25" ht="15.4">
       <c r="A5" t="s">
         <v>36</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>23.2</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.75">
+    <row r="6" spans="1:25" ht="15.4">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1959,7 +1959,7 @@
         <v>25.7</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="15.75">
+    <row r="7" spans="1:25" ht="15.4">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -2036,7 +2036,7 @@
         <v>25.8</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15.75">
+    <row r="8" spans="1:25" ht="15.4">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -2111,7 +2111,7 @@
         <v>24.4</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.75">
+    <row r="9" spans="1:25" ht="15.4">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -2188,7 +2188,7 @@
         <v>23.2</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="15.75">
+    <row r="10" spans="1:25" ht="15.4">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -2265,7 +2265,7 @@
         <v>15.3</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="15.75">
+    <row r="11" spans="1:25" ht="15.4">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -2298,7 +2298,7 @@
       <c r="X11" s="1"/>
       <c r="Y11" s="1"/>
     </row>
-    <row r="12" spans="1:25" ht="15.75">
+    <row r="12" spans="1:25" ht="15.4">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -2329,7 +2329,7 @@
       <c r="X12" s="1"/>
       <c r="Y12" s="1"/>
     </row>
-    <row r="13" spans="1:25" ht="15.75">
+    <row r="13" spans="1:25" ht="15.4">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -2406,7 +2406,7 @@
         <v>14.3</v>
       </c>
     </row>
-    <row r="14" spans="1:25" ht="15.75">
+    <row r="14" spans="1:25" ht="15.4">
       <c r="A14" t="s">
         <v>41</v>
       </c>
@@ -2437,7 +2437,7 @@
         <v>10.9</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="15.75">
+    <row r="15" spans="1:25" ht="15.4">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -2478,7 +2478,7 @@
         <v>10.9</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="15.75">
+    <row r="16" spans="1:25" ht="15.4">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -2553,7 +2553,7 @@
       </c>
       <c r="Y16" s="1"/>
     </row>
-    <row r="17" spans="1:25" ht="15.75">
+    <row r="17" spans="1:25" ht="15.4">
       <c r="A17" t="s">
         <v>42</v>
       </c>
@@ -2626,7 +2626,7 @@
         <v>14.3</v>
       </c>
     </row>
-    <row r="18" spans="1:25" ht="15.75">
+    <row r="18" spans="1:25" ht="15.4">
       <c r="A18" t="s">
         <v>46</v>
       </c>
@@ -2691,7 +2691,7 @@
       <c r="X18" s="1"/>
       <c r="Y18" s="1"/>
     </row>
-    <row r="19" spans="1:25" ht="15.75">
+    <row r="19" spans="1:25" ht="15.4">
       <c r="A19" t="s">
         <v>38</v>
       </c>
@@ -2768,7 +2768,7 @@
         <v>11.9</v>
       </c>
     </row>
-    <row r="20" spans="1:25" ht="15.75">
+    <row r="20" spans="1:25" ht="15.4">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -2845,7 +2845,7 @@
         <v>11.8</v>
       </c>
     </row>
-    <row r="21" spans="1:25" ht="15.75">
+    <row r="21" spans="1:25" ht="15.4">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -2922,7 +2922,7 @@
         <v>11.8</v>
       </c>
     </row>
-    <row r="22" spans="1:25" ht="15.75">
+    <row r="22" spans="1:25" ht="15.4">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -2999,7 +2999,7 @@
         <v>8.6</v>
       </c>
     </row>
-    <row r="23" spans="1:25" ht="15.75">
+    <row r="23" spans="1:25" ht="15.4">
       <c r="A23" t="s">
         <v>43</v>
       </c>
@@ -3076,7 +3076,7 @@
         <v>9.6</v>
       </c>
     </row>
-    <row r="24" spans="1:25" ht="15.75">
+    <row r="24" spans="1:25" ht="15.4">
       <c r="A24" t="s">
         <v>44</v>
       </c>
@@ -3153,7 +3153,7 @@
         <v>7.1</v>
       </c>
     </row>
-    <row r="25" spans="1:25" ht="15.75">
+    <row r="25" spans="1:25" ht="15.4">
       <c r="A25" t="s">
         <v>35</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>7.4</v>
       </c>
     </row>
-    <row r="26" spans="1:25" ht="15.75">
+    <row r="26" spans="1:25" ht="15.4">
       <c r="A26" t="s">
         <v>45</v>
       </c>
@@ -3267,10 +3267,10 @@
   <sheetPr>
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:Y24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:Y22"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25">
@@ -3347,7 +3347,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="15.75">
+    <row r="2" spans="1:25" ht="15.4">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -3424,7 +3424,7 @@
         <v>30.3</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15.75">
+    <row r="3" spans="1:25" ht="15.4">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -3501,7 +3501,7 @@
         <v>30.1</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.75">
+    <row r="4" spans="1:25" ht="15.4">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -3578,7 +3578,7 @@
         <v>25.1</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="15.75">
+    <row r="5" spans="1:25" ht="15.4">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -3655,7 +3655,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.75">
+    <row r="6" spans="1:25" ht="15.4">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -3732,7 +3732,7 @@
         <v>21.9</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="15.75">
+    <row r="7" spans="1:25" ht="15.4">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -3809,7 +3809,7 @@
         <v>23.7</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15.75">
+    <row r="8" spans="1:25" ht="15.4">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -3819,30 +3819,74 @@
       <c r="C8" s="1">
         <v>17.399999999999999</v>
       </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
-      <c r="Q8" s="1"/>
-      <c r="R8" s="1"/>
-      <c r="S8" s="1"/>
-      <c r="T8" s="1"/>
-      <c r="U8" s="1"/>
-      <c r="V8" s="1"/>
-      <c r="W8" s="1"/>
-      <c r="X8" s="1"/>
-      <c r="Y8" s="1"/>
-    </row>
-    <row r="9" spans="1:25" ht="15.75">
+      <c r="D8" s="1">
+        <v>8.4</v>
+      </c>
+      <c r="E8" s="1">
+        <v>7.8</v>
+      </c>
+      <c r="F8" s="1">
+        <v>7.2</v>
+      </c>
+      <c r="G8" s="1">
+        <v>6.6</v>
+      </c>
+      <c r="H8" s="1">
+        <v>6</v>
+      </c>
+      <c r="I8" s="1">
+        <v>5.4</v>
+      </c>
+      <c r="J8" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="K8" s="1">
+        <v>5.4</v>
+      </c>
+      <c r="L8" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="M8" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="N8" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="O8" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="P8" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="Q8" s="1">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="R8" s="1">
+        <v>5.3</v>
+      </c>
+      <c r="S8" s="1">
+        <v>5.9</v>
+      </c>
+      <c r="T8" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="U8" s="1">
+        <v>7.1</v>
+      </c>
+      <c r="V8" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="W8" s="1">
+        <v>5.9</v>
+      </c>
+      <c r="X8" s="1">
+        <v>5.3</v>
+      </c>
+      <c r="Y8" s="1">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" ht="15.4">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -3919,12 +3963,16 @@
         <v>18.100000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="15.75">
+    <row r="10" spans="1:25" ht="15.4">
       <c r="A10" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
+      <c r="B10" s="1">
+        <v>9.6</v>
+      </c>
+      <c r="C10" s="1">
+        <v>9</v>
+      </c>
       <c r="D10" s="1">
         <v>16.8</v>
       </c>
@@ -3992,7 +4040,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="15.75">
+    <row r="11" spans="1:25" ht="15.4">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -4069,731 +4117,767 @@
         <v>12.6</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="15.75">
+    <row r="12" spans="1:25" ht="15.4">
       <c r="A12" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="B12" s="1">
+        <v>8.1</v>
+      </c>
+      <c r="C12" s="1">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="D12" s="1">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="E12" s="1">
+        <v>9.9</v>
+      </c>
+      <c r="F12" s="1">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="G12" s="1">
+        <v>9.1</v>
+      </c>
+      <c r="H12" s="1">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="I12" s="1">
+        <v>9.5</v>
+      </c>
+      <c r="J12" s="1">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="K12" s="1">
+        <v>9.1</v>
+      </c>
+      <c r="L12" s="1">
+        <v>8.5</v>
+      </c>
+      <c r="M12" s="1">
+        <v>7.9</v>
+      </c>
+      <c r="N12" s="1">
+        <v>8.5</v>
+      </c>
+      <c r="O12" s="1">
+        <v>9.1</v>
+      </c>
+      <c r="P12" s="1">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>10.3</v>
+      </c>
+      <c r="R12" s="1">
+        <v>10.5</v>
+      </c>
+      <c r="S12" s="1">
+        <v>9.9</v>
+      </c>
+      <c r="T12" s="1">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="U12" s="1">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="V12" s="1">
+        <v>8.5</v>
+      </c>
+      <c r="W12" s="1">
+        <v>7.9</v>
+      </c>
+      <c r="X12" s="1">
+        <v>7.3</v>
+      </c>
+      <c r="Y12" s="1">
+        <v>6.7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25" ht="15.4">
+      <c r="A13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="1">
+        <v>13.1</v>
+      </c>
+      <c r="C13" s="1">
+        <v>12.5</v>
+      </c>
+      <c r="D13" s="1">
+        <v>11.9</v>
+      </c>
+      <c r="E13" s="1">
+        <v>11.3</v>
+      </c>
+      <c r="F13" s="1">
+        <v>10.7</v>
+      </c>
+      <c r="G13" s="1">
+        <v>10.1</v>
+      </c>
+      <c r="H13" s="1">
+        <v>9.5</v>
+      </c>
+      <c r="I13" s="1">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="J13" s="1">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="K13" s="1">
+        <v>8.5</v>
+      </c>
+      <c r="L13" s="1">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="M13" s="1">
+        <v>7.7</v>
+      </c>
+      <c r="N13" s="1">
+        <v>7.1</v>
+      </c>
+      <c r="O13" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="P13" s="1">
+        <v>5.9</v>
+      </c>
+      <c r="Q13" s="1">
+        <v>5.7</v>
+      </c>
+      <c r="R13" s="1">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="S13" s="1">
+        <v>5.7</v>
+      </c>
+      <c r="T13" s="1">
+        <v>6.3</v>
+      </c>
+      <c r="U13" s="1">
+        <v>6.9</v>
+      </c>
+      <c r="V13" s="1">
+        <v>6.3</v>
+      </c>
+      <c r="W13" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="X13" s="1">
+        <v>7.1</v>
+      </c>
+      <c r="Y13" s="1">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" ht="15.4">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="1">
+        <v>7.3</v>
+      </c>
+      <c r="C14" s="1">
+        <v>7.5</v>
+      </c>
+      <c r="D14" s="1">
+        <v>8.1</v>
+      </c>
+      <c r="E14" s="1">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="F14" s="1">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="G14" s="1">
+        <v>9.1</v>
+      </c>
+      <c r="H14" s="1">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="I14" s="1">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="J14" s="1">
+        <v>8.1</v>
+      </c>
+      <c r="K14" s="1">
+        <v>7.5</v>
+      </c>
+      <c r="L14" s="1">
+        <v>7.7</v>
+      </c>
+      <c r="M14" s="1">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="N14" s="1">
+        <v>8.9</v>
+      </c>
+      <c r="O14" s="1">
+        <v>9.1</v>
+      </c>
+      <c r="P14" s="1">
+        <v>8.5</v>
+      </c>
+      <c r="Q14" s="1">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="R14" s="1">
+        <v>8.5</v>
+      </c>
+      <c r="S14" s="1">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="T14" s="1">
+        <v>7.7</v>
+      </c>
+      <c r="U14" s="1">
+        <v>7.1</v>
+      </c>
+      <c r="V14" s="1">
+        <v>6.5</v>
+      </c>
+      <c r="W14" s="1">
+        <v>6.7</v>
+      </c>
+      <c r="X14" s="1">
+        <v>7.3</v>
+      </c>
+      <c r="Y14" s="1">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" ht="15.4">
+      <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="1">
+        <v>6.7</v>
+      </c>
+      <c r="C15" s="1">
+        <v>6.1</v>
+      </c>
+      <c r="D15" s="1">
+        <v>6.7</v>
+      </c>
+      <c r="E15" s="1">
+        <v>7.3</v>
+      </c>
+      <c r="F15" s="1">
+        <v>7.9</v>
+      </c>
+      <c r="G15" s="1">
+        <v>8.5</v>
+      </c>
+      <c r="H15" s="1">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="I15" s="1">
+        <v>8.1</v>
+      </c>
+      <c r="J15" s="1">
+        <v>7.5</v>
+      </c>
+      <c r="K15" s="1">
+        <v>6.9</v>
+      </c>
+      <c r="L15" s="1">
+        <v>6.7</v>
+      </c>
+      <c r="M15" s="1">
+        <v>6.9</v>
+      </c>
+      <c r="N15" s="1">
+        <v>7.5</v>
+      </c>
+      <c r="O15" s="1">
+        <v>8.1</v>
+      </c>
+      <c r="P15" s="1">
+        <v>7.5</v>
+      </c>
+      <c r="Q15" s="1">
+        <v>7.3</v>
+      </c>
+      <c r="R15" s="1">
+        <v>6.7</v>
+      </c>
+      <c r="S15" s="1">
+        <v>7.3</v>
+      </c>
+      <c r="T15" s="1">
+        <v>7.1</v>
+      </c>
+      <c r="U15" s="1">
+        <v>7.7</v>
+      </c>
+      <c r="V15" s="1">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="W15" s="1">
+        <v>8.9</v>
+      </c>
+      <c r="X15" s="1">
+        <v>9.5</v>
+      </c>
+      <c r="Y15" s="1">
+        <v>9.3000000000000007</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" ht="15.4">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="1">
+        <v>6.4</v>
+      </c>
+      <c r="C16" s="1">
+        <v>7</v>
+      </c>
+      <c r="D16" s="1">
+        <v>7.6</v>
+      </c>
+      <c r="E16" s="1">
+        <v>7.8</v>
+      </c>
+      <c r="F16" s="1">
+        <v>7.2</v>
+      </c>
+      <c r="G16" s="1">
+        <v>6.6</v>
+      </c>
+      <c r="H16" s="1">
+        <v>6</v>
+      </c>
+      <c r="I16" s="1">
+        <v>6.2</v>
+      </c>
+      <c r="J16" s="1">
+        <v>6</v>
+      </c>
+      <c r="K16" s="1">
+        <v>6.6</v>
+      </c>
+      <c r="L16" s="1">
+        <v>7.2</v>
+      </c>
+      <c r="M16" s="1">
+        <v>7.8</v>
+      </c>
+      <c r="N16" s="1">
+        <v>8.4</v>
+      </c>
+      <c r="O16" s="1">
+        <v>9</v>
+      </c>
+      <c r="P16" s="1">
         <v>9.6</v>
       </c>
-      <c r="C12" s="1">
-        <v>9</v>
-      </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
-      <c r="P12" s="1"/>
-      <c r="Q12" s="1"/>
-      <c r="R12" s="1"/>
-      <c r="S12" s="1"/>
-      <c r="T12" s="1"/>
-      <c r="U12" s="1"/>
-      <c r="V12" s="1"/>
-      <c r="W12" s="1"/>
-      <c r="X12" s="1"/>
-      <c r="Y12" s="1"/>
-    </row>
-    <row r="13" spans="1:25" ht="15.75">
-      <c r="A13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="1">
+      <c r="Q16" s="1">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="R16" s="1">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="S16" s="1">
+        <v>8.6</v>
+      </c>
+      <c r="T16" s="1">
+        <v>8</v>
+      </c>
+      <c r="U16" s="1">
+        <v>7.4</v>
+      </c>
+      <c r="V16" s="1">
+        <v>6.8</v>
+      </c>
+      <c r="W16" s="1">
+        <v>6.2</v>
+      </c>
+      <c r="X16" s="1">
+        <v>5.6</v>
+      </c>
+      <c r="Y16" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:25" ht="15.4">
+      <c r="A17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B17" s="1">
+        <v>11.8</v>
+      </c>
+      <c r="C17" s="1">
+        <v>11.2</v>
+      </c>
+      <c r="D17" s="1">
+        <v>10.6</v>
+      </c>
+      <c r="E17" s="1">
+        <v>10</v>
+      </c>
+      <c r="F17" s="1">
+        <v>9.4</v>
+      </c>
+      <c r="G17" s="1">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="H17" s="1">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="I17" s="1">
+        <v>7.6</v>
+      </c>
+      <c r="J17" s="1">
+        <v>7</v>
+      </c>
+      <c r="K17" s="1">
+        <v>6.4</v>
+      </c>
+      <c r="L17" s="1">
+        <v>5.8</v>
+      </c>
+      <c r="M17" s="1">
+        <v>6</v>
+      </c>
+      <c r="N17" s="1">
+        <v>6.6</v>
+      </c>
+      <c r="O17" s="1">
+        <v>6</v>
+      </c>
+      <c r="P17" s="1">
+        <v>5.4</v>
+      </c>
+      <c r="Q17" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="R17" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="S17" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="T17" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="U17" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="V17" s="1">
+        <v>4.7</v>
+      </c>
+      <c r="W17" s="1">
+        <v>5.3</v>
+      </c>
+      <c r="X17" s="1">
+        <v>5.9</v>
+      </c>
+      <c r="Y17" s="1">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:25" ht="15.4">
+      <c r="A18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="1">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="C18" s="1">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="D18" s="1">
+        <v>7.6</v>
+      </c>
+      <c r="E18" s="1">
+        <v>7</v>
+      </c>
+      <c r="F18" s="1">
+        <v>6.4</v>
+      </c>
+      <c r="G18" s="1">
+        <v>6.2</v>
+      </c>
+      <c r="H18" s="1">
+        <v>5.6</v>
+      </c>
+      <c r="I18" s="1">
+        <v>5</v>
+      </c>
+      <c r="J18" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="K18" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="L18" s="1">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="M18" s="1">
+        <v>5.7</v>
+      </c>
+      <c r="N18" s="1">
+        <v>6.3</v>
+      </c>
+      <c r="O18" s="1">
+        <v>6.9</v>
+      </c>
+      <c r="P18" s="1">
+        <v>7.5</v>
+      </c>
+      <c r="Q18" s="1">
         <v>8.1</v>
       </c>
-      <c r="C13" s="1">
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="D13" s="1">
-        <v>9.3000000000000007</v>
-      </c>
-      <c r="E13" s="1">
-        <v>9.9</v>
-      </c>
-      <c r="F13" s="1">
-        <v>9.6999999999999993</v>
-      </c>
-      <c r="G13" s="1">
-        <v>9.1</v>
-      </c>
-      <c r="H13" s="1">
-        <v>9.6999999999999993</v>
-      </c>
-      <c r="I13" s="1">
-        <v>9.5</v>
-      </c>
-      <c r="J13" s="1">
-        <v>9.6999999999999993</v>
-      </c>
-      <c r="K13" s="1">
-        <v>9.1</v>
-      </c>
-      <c r="L13" s="1">
-        <v>8.5</v>
-      </c>
-      <c r="M13" s="1">
+      <c r="R18" s="1">
         <v>7.9</v>
       </c>
-      <c r="N13" s="1">
-        <v>8.5</v>
-      </c>
-      <c r="O13" s="1">
-        <v>9.1</v>
-      </c>
-      <c r="P13" s="1">
-        <v>9.6999999999999993</v>
-      </c>
-      <c r="Q13" s="1">
-        <v>10.3</v>
-      </c>
-      <c r="R13" s="1">
-        <v>10.5</v>
-      </c>
-      <c r="S13" s="1">
-        <v>9.9</v>
-      </c>
-      <c r="T13" s="1">
-        <v>9.3000000000000007</v>
-      </c>
-      <c r="U13" s="1">
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="V13" s="1">
-        <v>8.5</v>
-      </c>
-      <c r="W13" s="1">
-        <v>7.9</v>
-      </c>
-      <c r="X13" s="1">
+      <c r="S18" s="1">
         <v>7.3</v>
       </c>
-      <c r="Y13" s="1">
+      <c r="T18" s="1">
         <v>6.7</v>
       </c>
-    </row>
-    <row r="14" spans="1:25" ht="15.75">
-      <c r="A14" t="s">
-        <v>25</v>
-      </c>
-      <c r="B14" s="1">
-        <v>13.1</v>
-      </c>
-      <c r="C14" s="1">
-        <v>12.5</v>
-      </c>
-      <c r="D14" s="1">
-        <v>11.9</v>
-      </c>
-      <c r="E14" s="1">
-        <v>11.3</v>
-      </c>
-      <c r="F14" s="1">
-        <v>10.7</v>
-      </c>
-      <c r="G14" s="1">
-        <v>10.1</v>
-      </c>
-      <c r="H14" s="1">
-        <v>9.5</v>
-      </c>
-      <c r="I14" s="1">
-        <v>9.3000000000000007</v>
-      </c>
-      <c r="J14" s="1">
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="K14" s="1">
-        <v>8.5</v>
-      </c>
-      <c r="L14" s="1">
-        <v>8.3000000000000007</v>
-      </c>
-      <c r="M14" s="1">
-        <v>7.7</v>
-      </c>
-      <c r="N14" s="1">
+      <c r="U18" s="1">
+        <v>6.1</v>
+      </c>
+      <c r="V18" s="1">
+        <v>5.5</v>
+      </c>
+      <c r="W18" s="1">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="X18" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="Y18" s="1">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:25" ht="15.4">
+      <c r="A19" t="s">
+        <v>41</v>
+      </c>
+      <c r="B19" s="1">
+        <v>7.2</v>
+      </c>
+      <c r="C19" s="1">
+        <v>6.6</v>
+      </c>
+      <c r="D19" s="1">
+        <v>6</v>
+      </c>
+      <c r="E19" s="1">
+        <v>5.4</v>
+      </c>
+      <c r="F19" s="1">
+        <v>5.6</v>
+      </c>
+      <c r="G19" s="1">
+        <v>5</v>
+      </c>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
+      <c r="P19" s="1"/>
+      <c r="Q19" s="1"/>
+      <c r="R19" s="1"/>
+      <c r="S19" s="1"/>
+      <c r="T19" s="1"/>
+      <c r="U19" s="1"/>
+      <c r="V19" s="1"/>
+      <c r="W19" s="1"/>
+      <c r="X19" s="1"/>
+      <c r="Y19" s="1"/>
+    </row>
+    <row r="20" spans="1:25" ht="15.4">
+      <c r="A20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="1">
+        <v>6.2</v>
+      </c>
+      <c r="C20" s="1">
+        <v>5.6</v>
+      </c>
+      <c r="D20" s="1">
+        <v>5</v>
+      </c>
+      <c r="E20" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="F20" s="1">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="G20" s="1">
+        <v>5.7</v>
+      </c>
+      <c r="H20" s="1">
+        <v>5.5</v>
+      </c>
+      <c r="I20" s="1">
+        <v>5.3</v>
+      </c>
+      <c r="J20" s="1">
+        <v>5.5</v>
+      </c>
+      <c r="K20" s="1">
+        <v>6.1</v>
+      </c>
+      <c r="L20" s="1">
+        <v>6.7</v>
+      </c>
+      <c r="M20" s="1">
+        <v>6.9</v>
+      </c>
+      <c r="N20" s="1">
+        <v>6.3</v>
+      </c>
+      <c r="O20" s="1">
+        <v>5.7</v>
+      </c>
+      <c r="P20" s="1">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="Q20" s="1">
+        <v>5.7</v>
+      </c>
+      <c r="R20" s="1">
+        <v>6.3</v>
+      </c>
+      <c r="S20" s="1">
+        <v>6.9</v>
+      </c>
+      <c r="T20" s="1">
         <v>7.1</v>
       </c>
-      <c r="O14" s="1">
+      <c r="U20" s="1">
         <v>6.5</v>
       </c>
-      <c r="P14" s="1">
+      <c r="V20" s="1">
         <v>5.9</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="W20" s="1">
         <v>5.7</v>
       </c>
-      <c r="R14" s="1">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="S14" s="1">
-        <v>5.7</v>
-      </c>
-      <c r="T14" s="1">
+      <c r="X20" s="1">
         <v>6.3</v>
       </c>
-      <c r="U14" s="1">
+      <c r="Y20" s="1">
         <v>6.9</v>
       </c>
-      <c r="V14" s="1">
-        <v>6.3</v>
-      </c>
-      <c r="W14" s="1">
-        <v>6.5</v>
-      </c>
-      <c r="X14" s="1">
-        <v>7.1</v>
-      </c>
-      <c r="Y14" s="1">
-        <v>7.7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:25" ht="15.75">
-      <c r="A15" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="1">
-        <v>7.3</v>
-      </c>
-      <c r="C15" s="1">
-        <v>7.5</v>
-      </c>
-      <c r="D15" s="1">
-        <v>8.1</v>
-      </c>
-      <c r="E15" s="1">
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="F15" s="1">
-        <v>9.3000000000000007</v>
-      </c>
-      <c r="G15" s="1">
-        <v>9.1</v>
-      </c>
-      <c r="H15" s="1">
-        <v>9.3000000000000007</v>
-      </c>
-      <c r="I15" s="1">
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="J15" s="1">
-        <v>8.1</v>
-      </c>
-      <c r="K15" s="1">
-        <v>7.5</v>
-      </c>
-      <c r="L15" s="1">
-        <v>7.7</v>
-      </c>
-      <c r="M15" s="1">
-        <v>8.3000000000000007</v>
-      </c>
-      <c r="N15" s="1">
-        <v>8.9</v>
-      </c>
-      <c r="O15" s="1">
-        <v>9.1</v>
-      </c>
-      <c r="P15" s="1">
-        <v>8.5</v>
-      </c>
-      <c r="Q15" s="1">
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="R15" s="1">
-        <v>8.5</v>
-      </c>
-      <c r="S15" s="1">
-        <v>8.3000000000000007</v>
-      </c>
-      <c r="T15" s="1">
-        <v>7.7</v>
-      </c>
-      <c r="U15" s="1">
-        <v>7.1</v>
-      </c>
-      <c r="V15" s="1">
-        <v>6.5</v>
-      </c>
-      <c r="W15" s="1">
-        <v>6.7</v>
-      </c>
-      <c r="X15" s="1">
-        <v>7.3</v>
-      </c>
-      <c r="Y15" s="1">
-        <v>7.9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:25" ht="15.75">
-      <c r="A16" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16" s="1">
-        <v>6.7</v>
-      </c>
-      <c r="C16" s="1">
-        <v>6.1</v>
-      </c>
-      <c r="D16" s="1">
-        <v>6.7</v>
-      </c>
-      <c r="E16" s="1">
-        <v>7.3</v>
-      </c>
-      <c r="F16" s="1">
-        <v>7.9</v>
-      </c>
-      <c r="G16" s="1">
-        <v>8.5</v>
-      </c>
-      <c r="H16" s="1">
-        <v>8.6999999999999993</v>
-      </c>
-      <c r="I16" s="1">
-        <v>8.1</v>
-      </c>
-      <c r="J16" s="1">
-        <v>7.5</v>
-      </c>
-      <c r="K16" s="1">
-        <v>6.9</v>
-      </c>
-      <c r="L16" s="1">
-        <v>6.7</v>
-      </c>
-      <c r="M16" s="1">
-        <v>6.9</v>
-      </c>
-      <c r="N16" s="1">
-        <v>7.5</v>
-      </c>
-      <c r="O16" s="1">
-        <v>8.1</v>
-      </c>
-      <c r="P16" s="1">
-        <v>7.5</v>
-      </c>
-      <c r="Q16" s="1">
-        <v>7.3</v>
-      </c>
-      <c r="R16" s="1">
-        <v>6.7</v>
-      </c>
-      <c r="S16" s="1">
-        <v>7.3</v>
-      </c>
-      <c r="T16" s="1">
-        <v>7.1</v>
-      </c>
-      <c r="U16" s="1">
-        <v>7.7</v>
-      </c>
-      <c r="V16" s="1">
-        <v>8.3000000000000007</v>
-      </c>
-      <c r="W16" s="1">
-        <v>8.9</v>
-      </c>
-      <c r="X16" s="1">
-        <v>9.5</v>
-      </c>
-      <c r="Y16" s="1">
-        <v>9.3000000000000007</v>
-      </c>
-    </row>
-    <row r="17" spans="1:25" ht="15.75">
-      <c r="A17" t="s">
-        <v>31</v>
-      </c>
-      <c r="B17" s="1">
-        <v>6.4</v>
-      </c>
-      <c r="C17" s="1">
-        <v>7</v>
-      </c>
-      <c r="D17" s="1">
-        <v>7.6</v>
-      </c>
-      <c r="E17" s="1">
-        <v>7.8</v>
-      </c>
-      <c r="F17" s="1">
-        <v>7.2</v>
-      </c>
-      <c r="G17" s="1">
-        <v>6.6</v>
-      </c>
-      <c r="H17" s="1">
+    </row>
+    <row r="21" spans="1:25" ht="15.4">
+      <c r="A21" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" s="1">
         <v>6</v>
       </c>
-      <c r="I17" s="1">
-        <v>6.2</v>
-      </c>
-      <c r="J17" s="1">
-        <v>6</v>
-      </c>
-      <c r="K17" s="1">
-        <v>6.6</v>
-      </c>
-      <c r="L17" s="1">
-        <v>7.2</v>
-      </c>
-      <c r="M17" s="1">
-        <v>7.8</v>
-      </c>
-      <c r="N17" s="1">
-        <v>8.4</v>
-      </c>
-      <c r="O17" s="1">
-        <v>9</v>
-      </c>
-      <c r="P17" s="1">
-        <v>9.6</v>
-      </c>
-      <c r="Q17" s="1">
-        <v>9.8000000000000007</v>
-      </c>
-      <c r="R17" s="1">
-        <v>9.1999999999999993</v>
-      </c>
-      <c r="S17" s="1">
-        <v>8.6</v>
-      </c>
-      <c r="T17" s="1">
-        <v>8</v>
-      </c>
-      <c r="U17" s="1">
-        <v>7.4</v>
-      </c>
-      <c r="V17" s="1">
-        <v>6.8</v>
-      </c>
-      <c r="W17" s="1">
-        <v>6.2</v>
-      </c>
-      <c r="X17" s="1">
-        <v>5.6</v>
-      </c>
-      <c r="Y17" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:25" ht="15.75">
-      <c r="A18" t="s">
-        <v>39</v>
-      </c>
-      <c r="B18" s="1">
-        <v>11.8</v>
-      </c>
-      <c r="C18" s="1">
-        <v>11.2</v>
-      </c>
-      <c r="D18" s="1">
-        <v>10.6</v>
-      </c>
-      <c r="E18" s="1">
-        <v>10</v>
-      </c>
-      <c r="F18" s="1">
-        <v>9.4</v>
-      </c>
-      <c r="G18" s="1">
-        <v>8.8000000000000007</v>
-      </c>
-      <c r="H18" s="1">
-        <v>8.1999999999999993</v>
-      </c>
-      <c r="I18" s="1">
-        <v>7.6</v>
-      </c>
-      <c r="J18" s="1">
-        <v>7</v>
-      </c>
-      <c r="K18" s="1">
-        <v>6.4</v>
-      </c>
-      <c r="L18" s="1">
-        <v>5.8</v>
-      </c>
-      <c r="M18" s="1">
-        <v>6</v>
-      </c>
-      <c r="N18" s="1">
-        <v>6.6</v>
-      </c>
-      <c r="O18" s="1">
-        <v>6</v>
-      </c>
-      <c r="P18" s="1">
+      <c r="C21" s="1">
         <v>5.4</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="D21" s="1">
         <v>4.8</v>
-      </c>
-      <c r="R18" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="S18" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="T18" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="U18" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="V18" s="1">
-        <v>4.7</v>
-      </c>
-      <c r="W18" s="1">
-        <v>5.3</v>
-      </c>
-      <c r="X18" s="1">
-        <v>5.9</v>
-      </c>
-      <c r="Y18" s="1">
-        <v>6.5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:25" ht="15.75">
-      <c r="A19" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19" s="1">
-        <v>8.8000000000000007</v>
-      </c>
-      <c r="C19" s="1">
-        <v>8.1999999999999993</v>
-      </c>
-      <c r="D19" s="1">
-        <v>7.6</v>
-      </c>
-      <c r="E19" s="1">
-        <v>7</v>
-      </c>
-      <c r="F19" s="1">
-        <v>6.4</v>
-      </c>
-      <c r="G19" s="1">
-        <v>6.2</v>
-      </c>
-      <c r="H19" s="1">
-        <v>5.6</v>
-      </c>
-      <c r="I19" s="1">
-        <v>5</v>
-      </c>
-      <c r="J19" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="K19" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="L19" s="1">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="M19" s="1">
-        <v>5.7</v>
-      </c>
-      <c r="N19" s="1">
-        <v>6.3</v>
-      </c>
-      <c r="O19" s="1">
-        <v>6.9</v>
-      </c>
-      <c r="P19" s="1">
-        <v>7.5</v>
-      </c>
-      <c r="Q19" s="1">
-        <v>8.1</v>
-      </c>
-      <c r="R19" s="1">
-        <v>7.9</v>
-      </c>
-      <c r="S19" s="1">
-        <v>7.3</v>
-      </c>
-      <c r="T19" s="1">
-        <v>6.7</v>
-      </c>
-      <c r="U19" s="1">
-        <v>6.1</v>
-      </c>
-      <c r="V19" s="1">
-        <v>5.5</v>
-      </c>
-      <c r="W19" s="1">
-        <v>4.9000000000000004</v>
-      </c>
-      <c r="X19" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="Y19" s="1">
-        <v>4.7</v>
-      </c>
-    </row>
-    <row r="20" spans="1:25" ht="15.75">
-      <c r="A20" t="s">
-        <v>41</v>
-      </c>
-      <c r="B20" s="1">
-        <v>7.2</v>
-      </c>
-      <c r="C20" s="1">
-        <v>6.6</v>
-      </c>
-      <c r="D20" s="1">
-        <v>6</v>
-      </c>
-      <c r="E20" s="1">
-        <v>5.4</v>
-      </c>
-      <c r="F20" s="1">
-        <v>5.6</v>
-      </c>
-      <c r="G20" s="1">
-        <v>5</v>
-      </c>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
-      <c r="P20" s="1"/>
-      <c r="Q20" s="1"/>
-      <c r="R20" s="1"/>
-      <c r="S20" s="1"/>
-      <c r="T20" s="1"/>
-      <c r="U20" s="1"/>
-      <c r="V20" s="1"/>
-      <c r="W20" s="1"/>
-      <c r="X20" s="1"/>
-      <c r="Y20" s="1"/>
-    </row>
-    <row r="21" spans="1:25" ht="15.75">
-      <c r="A21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21" s="1">
-        <v>6.2</v>
-      </c>
-      <c r="C21" s="1">
-        <v>5.6</v>
-      </c>
-      <c r="D21" s="1">
-        <v>5</v>
       </c>
       <c r="E21" s="1">
         <v>4.5</v>
       </c>
       <c r="F21" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="G21" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="H21" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="I21" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="J21" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="K21" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="L21" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="M21" s="1">
         <v>5.0999999999999996</v>
       </c>
-      <c r="G21" s="1">
+      <c r="N21" s="1">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="O21" s="1">
+        <v>4.7</v>
+      </c>
+      <c r="P21" s="1">
+        <v>4.5</v>
+      </c>
+      <c r="Q21" s="1">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="R21" s="1">
         <v>5.7</v>
       </c>
-      <c r="H21" s="1">
+      <c r="S21" s="1">
+        <v>5.9</v>
+      </c>
+      <c r="T21" s="1">
+        <v>6.1</v>
+      </c>
+      <c r="U21" s="1">
+        <v>6.7</v>
+      </c>
+      <c r="V21" s="1">
+        <v>7.3</v>
+      </c>
+      <c r="W21" s="1">
+        <v>6.7</v>
+      </c>
+      <c r="X21" s="1">
+        <v>6.1</v>
+      </c>
+      <c r="Y21" s="1">
         <v>5.5</v>
       </c>
-      <c r="I21" s="1">
-        <v>5.3</v>
-      </c>
-      <c r="J21" s="1">
-        <v>5.5</v>
-      </c>
-      <c r="K21" s="1">
-        <v>6.1</v>
-      </c>
-      <c r="L21" s="1">
-        <v>6.7</v>
-      </c>
-      <c r="M21" s="1">
-        <v>6.9</v>
-      </c>
-      <c r="N21" s="1">
-        <v>6.3</v>
-      </c>
-      <c r="O21" s="1">
-        <v>5.7</v>
-      </c>
-      <c r="P21" s="1">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="Q21" s="1">
-        <v>5.7</v>
-      </c>
-      <c r="R21" s="1">
-        <v>6.3</v>
-      </c>
-      <c r="S21" s="1">
-        <v>6.9</v>
-      </c>
-      <c r="T21" s="1">
-        <v>7.1</v>
-      </c>
-      <c r="U21" s="1">
-        <v>6.5</v>
-      </c>
-      <c r="V21" s="1">
-        <v>5.9</v>
-      </c>
-      <c r="W21" s="1">
-        <v>5.7</v>
-      </c>
-      <c r="X21" s="1">
-        <v>6.3</v>
-      </c>
-      <c r="Y21" s="1">
-        <v>6.9</v>
-      </c>
-    </row>
-    <row r="22" spans="1:25" ht="15.75">
+    </row>
+    <row r="22" spans="1:25" ht="15.4">
       <c r="A22" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
-      <c r="D22" s="1">
-        <v>8.4</v>
-      </c>
-      <c r="E22" s="1">
-        <v>7.8</v>
-      </c>
-      <c r="F22" s="1">
-        <v>7.2</v>
-      </c>
-      <c r="G22" s="1">
-        <v>6.6</v>
-      </c>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
       <c r="H22" s="1">
-        <v>6</v>
+        <v>4.5</v>
       </c>
       <c r="I22" s="1">
-        <v>5.4</v>
+        <v>4.5</v>
       </c>
       <c r="J22" s="1">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="K22" s="1">
-        <v>5.4</v>
+        <v>4.5</v>
       </c>
       <c r="L22" s="1">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="M22" s="1">
-        <v>4.5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="N22" s="1">
         <v>4.5</v>
@@ -4805,172 +4889,30 @@
         <v>4.5</v>
       </c>
       <c r="Q22" s="1">
-        <v>5.0999999999999996</v>
+        <v>4.5</v>
       </c>
       <c r="R22" s="1">
-        <v>5.3</v>
+        <v>4.5</v>
       </c>
       <c r="S22" s="1">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="T22" s="1">
-        <v>6.5</v>
+        <v>4.5</v>
       </c>
       <c r="U22" s="1">
-        <v>7.1</v>
+        <v>4.5</v>
       </c>
       <c r="V22" s="1">
-        <v>6.5</v>
+        <v>4.7</v>
       </c>
       <c r="W22" s="1">
-        <v>5.9</v>
+        <v>4.5</v>
       </c>
       <c r="X22" s="1">
-        <v>5.3</v>
+        <v>4.5</v>
       </c>
       <c r="Y22" s="1">
-        <v>5.9</v>
-      </c>
-    </row>
-    <row r="23" spans="1:25" ht="15.75">
-      <c r="A23" t="s">
-        <v>33</v>
-      </c>
-      <c r="B23" s="1">
-        <v>6</v>
-      </c>
-      <c r="C23" s="1">
-        <v>5.4</v>
-      </c>
-      <c r="D23" s="1">
-        <v>4.8</v>
-      </c>
-      <c r="E23" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="F23" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="G23" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="H23" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="I23" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="J23" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="K23" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="L23" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="M23" s="1">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="N23" s="1">
-        <v>4.9000000000000004</v>
-      </c>
-      <c r="O23" s="1">
-        <v>4.7</v>
-      </c>
-      <c r="P23" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="Q23" s="1">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="R23" s="1">
-        <v>5.7</v>
-      </c>
-      <c r="S23" s="1">
-        <v>5.9</v>
-      </c>
-      <c r="T23" s="1">
-        <v>6.1</v>
-      </c>
-      <c r="U23" s="1">
-        <v>6.7</v>
-      </c>
-      <c r="V23" s="1">
-        <v>7.3</v>
-      </c>
-      <c r="W23" s="1">
-        <v>6.7</v>
-      </c>
-      <c r="X23" s="1">
-        <v>6.1</v>
-      </c>
-      <c r="Y23" s="1">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:25" ht="15.75">
-      <c r="A24" t="s">
-        <v>35</v>
-      </c>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="I24" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="J24" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="K24" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="L24" s="1">
-        <v>4.7</v>
-      </c>
-      <c r="M24" s="1">
-        <v>4.9000000000000004</v>
-      </c>
-      <c r="N24" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="O24" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="P24" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="Q24" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="R24" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="S24" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="T24" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="U24" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="V24" s="1">
-        <v>4.7</v>
-      </c>
-      <c r="W24" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="X24" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="Y24" s="1">
         <v>4.5</v>
       </c>
     </row>
@@ -4985,9 +4927,9 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -5193,7 +5135,7 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B13">
         <v>10</v>
@@ -5363,7 +5305,7 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="B23">
         <v>5.9</v>
@@ -5389,9 +5331,9 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:W23"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -5462,7 +5404,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="15.75">
+    <row r="2" spans="1:23" ht="15.4">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -5533,7 +5475,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="15.75">
+    <row r="3" spans="1:23" ht="15.4">
       <c r="A3" t="s">
         <v>36</v>
       </c>
@@ -5604,7 +5546,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="15.75">
+    <row r="4" spans="1:23" ht="15.4">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -5675,7 +5617,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="15.75">
+    <row r="5" spans="1:23" ht="15.4">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -5746,7 +5688,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="15.75">
+    <row r="6" spans="1:23" ht="15.4">
       <c r="A6" t="s">
         <v>40</v>
       </c>
@@ -5817,7 +5759,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:23" ht="15.75">
+    <row r="7" spans="1:23" ht="15.4">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -5888,7 +5830,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="15.75">
+    <row r="8" spans="1:23" ht="15.4">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -5959,7 +5901,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:23" ht="15.75">
+    <row r="9" spans="1:23" ht="15.4">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -6030,7 +5972,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="15.75">
+    <row r="10" spans="1:23" ht="15.4">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -6101,7 +6043,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="15.75">
+    <row r="11" spans="1:23" ht="15.4">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -6172,7 +6114,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="15.75">
+    <row r="12" spans="1:23" ht="15.4">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -6243,7 +6185,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="15.75">
+    <row r="13" spans="1:23" ht="15.4">
       <c r="A13" t="s">
         <v>38</v>
       </c>
@@ -6314,7 +6256,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="15.75">
+    <row r="14" spans="1:23" ht="15.4">
       <c r="A14" t="s">
         <v>46</v>
       </c>
@@ -6355,7 +6297,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="15.75">
+    <row r="15" spans="1:23" ht="15.4">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -6426,7 +6368,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="15.75">
+    <row r="16" spans="1:23" ht="15.4">
       <c r="A16" t="s">
         <v>26</v>
       </c>
@@ -6497,7 +6439,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="15.75">
+    <row r="17" spans="1:23" ht="15.4">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -6568,7 +6510,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:23" ht="15.75">
+    <row r="18" spans="1:23" ht="15.4">
       <c r="A18" t="s">
         <v>32</v>
       </c>
@@ -6605,7 +6547,7 @@
       <c r="V18" s="1"/>
       <c r="W18" s="1"/>
     </row>
-    <row r="19" spans="1:23" ht="15.75">
+    <row r="19" spans="1:23" ht="15.4">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -6676,7 +6618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:23" ht="15.75">
+    <row r="20" spans="1:23" ht="15.4">
       <c r="A20" t="s">
         <v>31</v>
       </c>
@@ -6747,7 +6689,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="21" spans="1:23" ht="15.75">
+    <row r="21" spans="1:23" ht="15.4">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -6794,7 +6736,7 @@
       <c r="V21" s="1"/>
       <c r="W21" s="1"/>
     </row>
-    <row r="22" spans="1:23" ht="15.75">
+    <row r="22" spans="1:23" ht="15.4">
       <c r="A22" t="s">
         <v>47</v>
       </c>
@@ -6865,7 +6807,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="15.75">
+    <row r="23" spans="1:23" ht="15.4">
       <c r="A23" t="s">
         <v>45</v>
       </c>
@@ -6947,9 +6889,9 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:Y26"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25">
@@ -7026,7 +6968,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="15.75">
+    <row r="2" spans="1:25" ht="15.4">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -7103,7 +7045,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15.75">
+    <row r="3" spans="1:25" ht="15.4">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -7180,7 +7122,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.75">
+    <row r="4" spans="1:25" ht="15.4">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -7257,7 +7199,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="15.75">
+    <row r="5" spans="1:25" ht="15.4">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -7288,7 +7230,7 @@
       <c r="X5" s="1"/>
       <c r="Y5" s="1"/>
     </row>
-    <row r="6" spans="1:25" ht="15.75">
+    <row r="6" spans="1:25" ht="15.4">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -7365,7 +7307,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="15.75">
+    <row r="7" spans="1:25" ht="15.4">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -7440,7 +7382,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15.75">
+    <row r="8" spans="1:25" ht="15.4">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -7517,7 +7459,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.75">
+    <row r="9" spans="1:25" ht="15.4">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -7594,7 +7536,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="15.75">
+    <row r="10" spans="1:25" ht="15.4">
       <c r="A10" t="s">
         <v>36</v>
       </c>
@@ -7671,7 +7613,7 @@
         <v>-18</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="15.75">
+    <row r="11" spans="1:25" ht="15.4">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -7704,7 +7646,7 @@
       <c r="X11" s="1"/>
       <c r="Y11" s="1"/>
     </row>
-    <row r="12" spans="1:25" ht="15.75">
+    <row r="12" spans="1:25" ht="15.4">
       <c r="A12" t="s">
         <v>41</v>
       </c>
@@ -7735,7 +7677,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:25" ht="15.75">
+    <row r="13" spans="1:25" ht="15.4">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -7808,7 +7750,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:25" ht="15.75">
+    <row r="14" spans="1:25" ht="15.4">
       <c r="A14" t="s">
         <v>40</v>
       </c>
@@ -7885,7 +7827,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="15.75">
+    <row r="15" spans="1:25" ht="15.4">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -7926,7 +7868,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="15.75">
+    <row r="16" spans="1:25" ht="15.4">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -8001,7 +7943,7 @@
       </c>
       <c r="Y16" s="1"/>
     </row>
-    <row r="17" spans="1:25" ht="15.75">
+    <row r="17" spans="1:25" ht="15.4">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -8078,7 +8020,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:25" ht="15.75">
+    <row r="18" spans="1:25" ht="15.4">
       <c r="A18" t="s">
         <v>46</v>
       </c>
@@ -8143,7 +8085,7 @@
       <c r="X18" s="1"/>
       <c r="Y18" s="1"/>
     </row>
-    <row r="19" spans="1:25" ht="15.75">
+    <row r="19" spans="1:25" ht="15.4">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -8220,7 +8162,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:25" ht="15.75">
+    <row r="20" spans="1:25" ht="15.4">
       <c r="A20" t="s">
         <v>28</v>
       </c>
@@ -8297,7 +8239,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:25" ht="15.75">
+    <row r="21" spans="1:25" ht="15.4">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -8374,7 +8316,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:25" ht="15.75">
+    <row r="22" spans="1:25" ht="15.4">
       <c r="A22" t="s">
         <v>38</v>
       </c>
@@ -8451,7 +8393,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:25" ht="15.75">
+    <row r="23" spans="1:25" ht="15.4">
       <c r="A23" t="s">
         <v>44</v>
       </c>
@@ -8528,7 +8470,7 @@
         <v>-16</v>
       </c>
     </row>
-    <row r="24" spans="1:25" ht="15.75">
+    <row r="24" spans="1:25" ht="15.4">
       <c r="A24" t="s">
         <v>35</v>
       </c>
@@ -8575,7 +8517,7 @@
         <v>-20</v>
       </c>
     </row>
-    <row r="25" spans="1:25" ht="15.75">
+    <row r="25" spans="1:25" ht="15.4">
       <c r="A25" t="s">
         <v>45</v>
       </c>
@@ -8632,7 +8574,7 @@
       <c r="X25" s="1"/>
       <c r="Y25" s="1"/>
     </row>
-    <row r="26" spans="1:25" ht="15.75">
+    <row r="26" spans="1:25" ht="15.4">
       <c r="A26" t="s">
         <v>26</v>
       </c>
@@ -8720,7 +8662,10 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:Y22"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="14.19921875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:25">
       <c r="B1">
@@ -10375,13 +10320,13 @@
   <sheetPr>
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:4">
       <c r="B1">
         <v>1</v>
       </c>
@@ -10391,11 +10336,8 @@
       <c r="D1">
         <v>3</v>
       </c>
-      <c r="E1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -10409,7 +10351,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -10423,7 +10365,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -10437,7 +10379,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -10451,7 +10393,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -10465,7 +10407,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -10479,7 +10421,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -10493,7 +10435,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -10507,7 +10449,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -10521,7 +10463,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:4">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -10535,7 +10477,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:4">
       <c r="A12" t="s">
         <v>26</v>
       </c>
@@ -10549,7 +10491,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:4">
       <c r="A13" t="s">
         <v>27</v>
       </c>
@@ -10563,7 +10505,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:4">
       <c r="A14" t="s">
         <v>28</v>
       </c>
@@ -10577,7 +10519,7 @@
         <v>-17</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:4">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -10591,7 +10533,7 @@
         <v>-14</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:4">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -10711,7 +10653,7 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{008844FF-9942-4BA0-9033-82ED2D862880}">
   <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" t="s">
@@ -10990,9 +10932,9 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:Y11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25">
@@ -11069,7 +11011,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="15.75">
+    <row r="2" spans="1:25" ht="15.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -11146,7 +11088,7 @@
         <v>29.7</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15.75">
+    <row r="3" spans="1:25" ht="15.4">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -11223,7 +11165,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.75">
+    <row r="4" spans="1:25" ht="15.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -11300,7 +11242,7 @@
         <v>25.3</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="15.75">
+    <row r="5" spans="1:25" ht="15.4">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -11377,7 +11319,7 @@
         <v>25.1</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.75">
+    <row r="6" spans="1:25" ht="15.4">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -11454,7 +11396,7 @@
         <v>14.4</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="15.75">
+    <row r="7" spans="1:25" ht="15.4">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -11531,7 +11473,7 @@
         <v>12.9</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15.75">
+    <row r="8" spans="1:25" ht="15.4">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -11608,7 +11550,7 @@
         <v>12.1</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.75">
+    <row r="9" spans="1:25" ht="15.4">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -11685,7 +11627,7 @@
         <v>12.2</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="15.75">
+    <row r="10" spans="1:25" ht="15.4">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -11762,7 +11704,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="15.75">
+    <row r="11" spans="1:25" ht="15.4">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -11850,7 +11792,7 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:Y11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" spans="1:25">
       <c r="B1">
@@ -11926,7 +11868,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="15.75">
+    <row r="2" spans="1:25" ht="15.4">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -12003,7 +11945,7 @@
         <v>36.1</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15.75">
+    <row r="3" spans="1:25" ht="15.4">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -12080,7 +12022,7 @@
         <v>31.8</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.75">
+    <row r="4" spans="1:25" ht="15.4">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -12157,7 +12099,7 @@
         <v>31.1</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="15.75">
+    <row r="5" spans="1:25" ht="15.4">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -12234,7 +12176,7 @@
         <v>28.4</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.75">
+    <row r="6" spans="1:25" ht="15.4">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -12311,7 +12253,7 @@
         <v>19.5</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="15.75">
+    <row r="7" spans="1:25" ht="15.4">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -12388,7 +12330,7 @@
         <v>16.2</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15.75">
+    <row r="8" spans="1:25" ht="15.4">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -12465,7 +12407,7 @@
         <v>15.6</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.75">
+    <row r="9" spans="1:25" ht="15.4">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -12542,7 +12484,7 @@
         <v>10.3</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="15.75">
+    <row r="10" spans="1:25" ht="15.4">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -12619,7 +12561,7 @@
         <v>10.1</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="15.75">
+    <row r="11" spans="1:25" ht="15.4">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -12707,7 +12649,7 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="B1">
@@ -12921,7 +12863,7 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="V1:AR11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" spans="22:44">
       <c r="W1">
@@ -12991,7 +12933,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="22:44" ht="15.75">
+    <row r="2" spans="22:44" ht="15.4">
       <c r="V2" t="s">
         <v>0</v>
       </c>
@@ -13062,7 +13004,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="22:44" ht="15.75">
+    <row r="3" spans="22:44" ht="15.4">
       <c r="V3" t="s">
         <v>2</v>
       </c>
@@ -13133,7 +13075,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="22:44" ht="15.75">
+    <row r="4" spans="22:44" ht="15.4">
       <c r="V4" t="s">
         <v>3</v>
       </c>
@@ -13204,7 +13146,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="22:44" ht="15.75">
+    <row r="5" spans="22:44" ht="15.4">
       <c r="V5" t="s">
         <v>4</v>
       </c>
@@ -13275,7 +13217,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="22:44" ht="15.75">
+    <row r="6" spans="22:44" ht="15.4">
       <c r="V6" t="s">
         <v>1</v>
       </c>
@@ -13346,7 +13288,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="22:44" ht="15.75">
+    <row r="7" spans="22:44" ht="15.4">
       <c r="V7" t="s">
         <v>5</v>
       </c>
@@ -13417,7 +13359,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="22:44" ht="15.75">
+    <row r="8" spans="22:44" ht="15.4">
       <c r="V8" t="s">
         <v>6</v>
       </c>
@@ -13488,7 +13430,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="22:44" ht="15.75">
+    <row r="9" spans="22:44" ht="15.4">
       <c r="V9" t="s">
         <v>7</v>
       </c>
@@ -13559,7 +13501,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="22:44" ht="15.75">
+    <row r="10" spans="22:44" ht="15.4">
       <c r="V10" t="s">
         <v>9</v>
       </c>
@@ -13630,7 +13572,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="22:44" ht="15.75">
+    <row r="11" spans="22:44" ht="15.4">
       <c r="V11" t="s">
         <v>8</v>
       </c>
@@ -13712,7 +13654,7 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:Y11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" spans="1:25">
       <c r="B1">
@@ -13788,7 +13730,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="15.75">
+    <row r="2" spans="1:25" ht="15.4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -13865,7 +13807,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15.75">
+    <row r="3" spans="1:25" ht="15.4">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -13942,7 +13884,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.75">
+    <row r="4" spans="1:25" ht="15.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -14019,7 +13961,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="15.75">
+    <row r="5" spans="1:25" ht="15.4">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -14096,7 +14038,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.75">
+    <row r="6" spans="1:25" ht="15.4">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -14173,7 +14115,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="15.75">
+    <row r="7" spans="1:25" ht="15.4">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -14250,7 +14192,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15.75">
+    <row r="8" spans="1:25" ht="15.4">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -14327,7 +14269,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.75">
+    <row r="9" spans="1:25" ht="15.4">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -14404,7 +14346,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="15.75">
+    <row r="10" spans="1:25" ht="15.4">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -14481,7 +14423,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="15.75">
+    <row r="11" spans="1:25" ht="15.4">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -14569,7 +14511,7 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="BR1:CP11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1" spans="70:94">
       <c r="BS1">
@@ -15425,13 +15367,13 @@
   <sheetPr>
     <tabColor theme="5"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:4">
       <c r="B1">
         <v>1</v>
       </c>
@@ -15441,11 +15383,8 @@
       <c r="D1">
         <v>3</v>
       </c>
-      <c r="E1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -15459,7 +15398,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -15473,7 +15412,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -15487,7 +15426,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -15501,7 +15440,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -15515,7 +15454,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:4">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -15529,7 +15468,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:4">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -15543,7 +15482,7 @@
         <v>-12</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:4">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -15557,7 +15496,7 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -15571,7 +15510,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:4">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -15585,7 +15524,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:4">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -15610,9 +15549,9 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:W23"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="18.75" customHeight="1">
@@ -15683,7 +15622,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="15.75">
+    <row r="2" spans="1:23" ht="15.4">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -15754,7 +15693,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="15.75">
+    <row r="3" spans="1:23" ht="15.4">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -15825,7 +15764,7 @@
         <v>25.3</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="15.75">
+    <row r="4" spans="1:23" ht="15.4">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -15896,7 +15835,7 @@
         <v>23.5</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="15.75">
+    <row r="5" spans="1:23" ht="15.4">
       <c r="A5" t="s">
         <v>36</v>
       </c>
@@ -15967,7 +15906,7 @@
         <v>20.8</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="15.75">
+    <row r="6" spans="1:23" ht="15.4">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -16038,7 +15977,7 @@
         <v>20.2</v>
       </c>
     </row>
-    <row r="7" spans="1:23" ht="15.75">
+    <row r="7" spans="1:23" ht="15.4">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -16109,7 +16048,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="15.75">
+    <row r="8" spans="1:23" ht="15.4">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -16180,7 +16119,7 @@
         <v>19.8</v>
       </c>
     </row>
-    <row r="9" spans="1:23" ht="15.75">
+    <row r="9" spans="1:23" ht="15.4">
       <c r="A9" t="s">
         <v>40</v>
       </c>
@@ -16251,7 +16190,7 @@
         <v>15.8</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="15.75">
+    <row r="10" spans="1:23" ht="15.4">
       <c r="A10" t="s">
         <v>30</v>
       </c>
@@ -16322,7 +16261,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="15.75">
+    <row r="11" spans="1:23" ht="15.4">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -16393,7 +16332,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="15.75">
+    <row r="12" spans="1:23" ht="15.4">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -16464,7 +16403,7 @@
         <v>15.4</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="15.75">
+    <row r="13" spans="1:23" ht="15.4">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -16535,7 +16474,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="15.75">
+    <row r="14" spans="1:23" ht="15.4">
       <c r="A14" t="s">
         <v>47</v>
       </c>
@@ -16606,7 +16545,7 @@
         <v>9.6</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="15.75">
+    <row r="15" spans="1:23" ht="15.4">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -16677,7 +16616,7 @@
         <v>11.3</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="15.75">
+    <row r="16" spans="1:23" ht="15.4">
       <c r="A16" t="s">
         <v>42</v>
       </c>
@@ -16748,7 +16687,7 @@
         <v>9.6</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="15.75">
+    <row r="17" spans="1:23" ht="15.4">
       <c r="A17" t="s">
         <v>43</v>
       </c>
@@ -16819,7 +16758,7 @@
         <v>7.7</v>
       </c>
     </row>
-    <row r="18" spans="1:23" ht="15.75">
+    <row r="18" spans="1:23" ht="15.4">
       <c r="A18" t="s">
         <v>38</v>
       </c>
@@ -16890,7 +16829,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="19" spans="1:23" ht="15.75">
+    <row r="19" spans="1:23" ht="15.4">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -16927,7 +16866,7 @@
       <c r="V19" s="1"/>
       <c r="W19" s="1"/>
     </row>
-    <row r="20" spans="1:23" ht="15.75">
+    <row r="20" spans="1:23" ht="15.4">
       <c r="A20" t="s">
         <v>46</v>
       </c>
@@ -16968,7 +16907,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="21" spans="1:23" ht="15.75">
+    <row r="21" spans="1:23" ht="15.4">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -17015,7 +16954,7 @@
       <c r="V21" s="1"/>
       <c r="W21" s="1"/>
     </row>
-    <row r="22" spans="1:23" ht="15.75">
+    <row r="22" spans="1:23" ht="15.4">
       <c r="A22" t="s">
         <v>31</v>
       </c>
@@ -17086,7 +17025,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="15.75">
+    <row r="23" spans="1:23" ht="15.4">
       <c r="A23" t="s">
         <v>45</v>
       </c>

</xml_diff>

<commit_message>
elo table added and tested
</commit_message>
<xml_diff>
--- a/data/raw/newHistPointAndPrice.xlsx
+++ b/data/raw/newHistPointAndPrice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44FF69F0-2F79-4E27-976C-C30B83A428A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1E27BF5-1AD3-40BB-A12E-136B99E4CE8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5700" yWindow="675" windowWidth="16200" windowHeight="9307" tabRatio="864" firstSheet="11" activeTab="15" xr2:uid="{2D04FC15-E09F-4251-B381-E10D89E9EC62}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" firstSheet="11" activeTab="14" xr2:uid="{2D04FC15-E09F-4251-B381-E10D89E9EC62}"/>
   </bookViews>
   <sheets>
     <sheet name="2023ConstructorPrice" sheetId="1" r:id="rId1"/>
@@ -689,9 +689,9 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:W11"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -762,7 +762,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="15.4">
+    <row r="2" spans="1:23" ht="15.75">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -833,7 +833,7 @@
         <v>29.7</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="15.4">
+    <row r="3" spans="1:23" ht="15.75">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -904,7 +904,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="15.4">
+    <row r="4" spans="1:23" ht="15.75">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -975,7 +975,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="15.4">
+    <row r="5" spans="1:23" ht="15.75">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1046,7 +1046,7 @@
         <v>17.100000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="15.4">
+    <row r="6" spans="1:23" ht="15.75">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1117,7 +1117,7 @@
         <v>14.2</v>
       </c>
     </row>
-    <row r="7" spans="1:23" ht="15.4">
+    <row r="7" spans="1:23" ht="15.75">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -1188,7 +1188,7 @@
         <v>13.4</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="15.4">
+    <row r="8" spans="1:23" ht="15.75">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1259,7 +1259,7 @@
         <v>8.6999999999999993</v>
       </c>
     </row>
-    <row r="9" spans="1:23" ht="15.4">
+    <row r="9" spans="1:23" ht="15.75">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1330,7 +1330,7 @@
         <v>6.6</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="15.4">
+    <row r="10" spans="1:23" ht="15.75">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1401,7 +1401,7 @@
         <v>7.8</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="15.4">
+    <row r="11" spans="1:23" ht="15.75">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1483,9 +1483,9 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:W23"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23">
@@ -1556,7 +1556,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="15.4">
+    <row r="2" spans="1:23" ht="15.75">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1627,7 +1627,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="15.4">
+    <row r="3" spans="1:23" ht="15.75">
       <c r="A3" t="s">
         <v>35</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="15.4">
+    <row r="4" spans="1:23" ht="15.75">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -1769,7 +1769,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="15.4">
+    <row r="5" spans="1:23" ht="15.75">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -1840,7 +1840,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="15.4">
+    <row r="6" spans="1:23" ht="15.75">
       <c r="A6" t="s">
         <v>37</v>
       </c>
@@ -1911,7 +1911,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:23" ht="15.4">
+    <row r="7" spans="1:23" ht="15.75">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -1982,7 +1982,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="15.4">
+    <row r="8" spans="1:23" ht="15.75">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -2053,7 +2053,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9" spans="1:23" ht="15.4">
+    <row r="9" spans="1:23" ht="15.75">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -2124,7 +2124,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="15.4">
+    <row r="10" spans="1:23" ht="15.75">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -2195,7 +2195,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="15.4">
+    <row r="11" spans="1:23" ht="15.75">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -2266,7 +2266,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="15.4">
+    <row r="12" spans="1:23" ht="15.75">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -2337,7 +2337,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="15.4">
+    <row r="13" spans="1:23" ht="15.75">
       <c r="A13" t="s">
         <v>36</v>
       </c>
@@ -2408,7 +2408,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="15.4">
+    <row r="14" spans="1:23" ht="15.75">
       <c r="A14" t="s">
         <v>42</v>
       </c>
@@ -2449,7 +2449,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="15.4">
+    <row r="15" spans="1:23" ht="15.75">
       <c r="A15" t="s">
         <v>79</v>
       </c>
@@ -2520,7 +2520,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="15.4">
+    <row r="16" spans="1:23" ht="15.75">
       <c r="A16" t="s">
         <v>26</v>
       </c>
@@ -2591,7 +2591,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="15.4">
+    <row r="17" spans="1:23" ht="15.75">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -2662,7 +2662,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:23" ht="15.4">
+    <row r="18" spans="1:23" ht="15.75">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -2699,7 +2699,7 @@
       <c r="V18" s="1"/>
       <c r="W18" s="1"/>
     </row>
-    <row r="19" spans="1:23" ht="15.4">
+    <row r="19" spans="1:23" ht="15.75">
       <c r="A19" t="s">
         <v>39</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:23" ht="15.4">
+    <row r="20" spans="1:23" ht="15.75">
       <c r="A20" t="s">
         <v>30</v>
       </c>
@@ -2841,7 +2841,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="21" spans="1:23" ht="15.4">
+    <row r="21" spans="1:23" ht="15.75">
       <c r="A21" t="s">
         <v>43</v>
       </c>
@@ -2888,7 +2888,7 @@
       <c r="V21" s="1"/>
       <c r="W21" s="1"/>
     </row>
-    <row r="22" spans="1:23" ht="15.4">
+    <row r="22" spans="1:23" ht="15.75">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -2959,7 +2959,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="15.4">
+    <row r="23" spans="1:23" ht="15.75">
       <c r="A23" t="s">
         <v>41</v>
       </c>
@@ -3041,9 +3041,9 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:Y26"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25">
@@ -3120,7 +3120,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="15.4">
+    <row r="2" spans="1:25" ht="15.75">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3197,7 +3197,7 @@
         <v>32.299999999999997</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15.4">
+    <row r="3" spans="1:25" ht="15.75">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -3274,7 +3274,7 @@
         <v>27.5</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.4">
+    <row r="4" spans="1:25" ht="15.75">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -3351,7 +3351,7 @@
         <v>26.1</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="15.4">
+    <row r="5" spans="1:25" ht="15.75">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -3428,7 +3428,7 @@
         <v>23.2</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.4">
+    <row r="6" spans="1:25" ht="15.75">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -3505,7 +3505,7 @@
         <v>25.7</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="15.4">
+    <row r="7" spans="1:25" ht="15.75">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -3582,7 +3582,7 @@
         <v>25.8</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15.4">
+    <row r="8" spans="1:25" ht="15.75">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -3657,7 +3657,7 @@
         <v>24.4</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.4">
+    <row r="9" spans="1:25" ht="15.75">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -3734,7 +3734,7 @@
         <v>23.2</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="15.4">
+    <row r="10" spans="1:25" ht="15.75">
       <c r="A10" t="s">
         <v>37</v>
       </c>
@@ -3811,7 +3811,7 @@
         <v>15.3</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="15.4">
+    <row r="11" spans="1:25" ht="15.75">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -3844,7 +3844,7 @@
       <c r="X11" s="1"/>
       <c r="Y11" s="1"/>
     </row>
-    <row r="12" spans="1:25" ht="15.4">
+    <row r="12" spans="1:25" ht="15.75">
       <c r="A12" t="s">
         <v>28</v>
       </c>
@@ -3875,7 +3875,7 @@
       <c r="X12" s="1"/>
       <c r="Y12" s="1"/>
     </row>
-    <row r="13" spans="1:25" ht="15.4">
+    <row r="13" spans="1:25" ht="15.75">
       <c r="A13" t="s">
         <v>27</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>14.3</v>
       </c>
     </row>
-    <row r="14" spans="1:25" ht="15.4">
+    <row r="14" spans="1:25" ht="15.75">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -3983,7 +3983,7 @@
         <v>10.9</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="15.4">
+    <row r="15" spans="1:25" ht="15.75">
       <c r="A15" t="s">
         <v>31</v>
       </c>
@@ -4024,7 +4024,7 @@
         <v>10.9</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="15.4">
+    <row r="16" spans="1:25" ht="15.75">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -4099,7 +4099,7 @@
       </c>
       <c r="Y16" s="1"/>
     </row>
-    <row r="17" spans="1:25" ht="15.4">
+    <row r="17" spans="1:25" ht="15.75">
       <c r="A17" t="s">
         <v>39</v>
       </c>
@@ -4172,7 +4172,7 @@
         <v>14.3</v>
       </c>
     </row>
-    <row r="18" spans="1:25" ht="15.4">
+    <row r="18" spans="1:25" ht="15.75">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -4237,7 +4237,7 @@
       <c r="X18" s="1"/>
       <c r="Y18" s="1"/>
     </row>
-    <row r="19" spans="1:25" ht="15.4">
+    <row r="19" spans="1:25" ht="15.75">
       <c r="A19" t="s">
         <v>36</v>
       </c>
@@ -4314,7 +4314,7 @@
         <v>11.9</v>
       </c>
     </row>
-    <row r="20" spans="1:25" ht="15.4">
+    <row r="20" spans="1:25" ht="15.75">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -4391,7 +4391,7 @@
         <v>11.8</v>
       </c>
     </row>
-    <row r="21" spans="1:25" ht="15.4">
+    <row r="21" spans="1:25" ht="15.75">
       <c r="A21" t="s">
         <v>30</v>
       </c>
@@ -4468,7 +4468,7 @@
         <v>11.8</v>
       </c>
     </row>
-    <row r="22" spans="1:25" ht="15.4">
+    <row r="22" spans="1:25" ht="15.75">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -4545,7 +4545,7 @@
         <v>8.6</v>
       </c>
     </row>
-    <row r="23" spans="1:25" ht="15.4">
+    <row r="23" spans="1:25" ht="15.75">
       <c r="A23" t="s">
         <v>79</v>
       </c>
@@ -4622,7 +4622,7 @@
         <v>9.6</v>
       </c>
     </row>
-    <row r="24" spans="1:25" ht="15.4">
+    <row r="24" spans="1:25" ht="15.75">
       <c r="A24" t="s">
         <v>40</v>
       </c>
@@ -4699,7 +4699,7 @@
         <v>7.1</v>
       </c>
     </row>
-    <row r="25" spans="1:25" ht="15.4">
+    <row r="25" spans="1:25" ht="15.75">
       <c r="A25" t="s">
         <v>34</v>
       </c>
@@ -4746,7 +4746,7 @@
         <v>7.4</v>
       </c>
     </row>
-    <row r="26" spans="1:25" ht="15.4">
+    <row r="26" spans="1:25" ht="15.75">
       <c r="A26" t="s">
         <v>41</v>
       </c>
@@ -4814,9 +4814,9 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:Y26"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25">
@@ -4893,7 +4893,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="15.4">
+    <row r="2" spans="1:25" ht="15.75">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -4970,7 +4970,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15.4">
+    <row r="3" spans="1:25" ht="15.75">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -5047,7 +5047,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.4">
+    <row r="4" spans="1:25" ht="15.75">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -5124,7 +5124,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="15.4">
+    <row r="5" spans="1:25" ht="15.75">
       <c r="A5" t="s">
         <v>28</v>
       </c>
@@ -5155,7 +5155,7 @@
       <c r="X5" s="1"/>
       <c r="Y5" s="1"/>
     </row>
-    <row r="6" spans="1:25" ht="15.4">
+    <row r="6" spans="1:25" ht="15.75">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -5232,7 +5232,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="15.4">
+    <row r="7" spans="1:25" ht="15.75">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -5307,7 +5307,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15.4">
+    <row r="8" spans="1:25" ht="15.75">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -5384,7 +5384,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.4">
+    <row r="9" spans="1:25" ht="15.75">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -5461,7 +5461,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="15.4">
+    <row r="10" spans="1:25" ht="15.75">
       <c r="A10" t="s">
         <v>35</v>
       </c>
@@ -5538,7 +5538,7 @@
         <v>-18</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="15.4">
+    <row r="11" spans="1:25" ht="15.75">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -5571,7 +5571,7 @@
       <c r="X11" s="1"/>
       <c r="Y11" s="1"/>
     </row>
-    <row r="12" spans="1:25" ht="15.4">
+    <row r="12" spans="1:25" ht="15.75">
       <c r="A12" t="s">
         <v>38</v>
       </c>
@@ -5602,7 +5602,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:25" ht="15.4">
+    <row r="13" spans="1:25" ht="15.75">
       <c r="A13" t="s">
         <v>39</v>
       </c>
@@ -5675,7 +5675,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:25" ht="15.4">
+    <row r="14" spans="1:25" ht="15.75">
       <c r="A14" t="s">
         <v>37</v>
       </c>
@@ -5752,7 +5752,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="15.4">
+    <row r="15" spans="1:25" ht="15.75">
       <c r="A15" t="s">
         <v>31</v>
       </c>
@@ -5793,7 +5793,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="15.4">
+    <row r="16" spans="1:25" ht="15.75">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -5868,7 +5868,7 @@
       </c>
       <c r="Y16" s="1"/>
     </row>
-    <row r="17" spans="1:25" ht="15.4">
+    <row r="17" spans="1:25" ht="15.75">
       <c r="A17" t="s">
         <v>79</v>
       </c>
@@ -5945,7 +5945,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:25" ht="15.4">
+    <row r="18" spans="1:25" ht="15.75">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -6010,7 +6010,7 @@
       <c r="X18" s="1"/>
       <c r="Y18" s="1"/>
     </row>
-    <row r="19" spans="1:25" ht="15.4">
+    <row r="19" spans="1:25" ht="15.75">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -6087,7 +6087,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="1:25" ht="15.4">
+    <row r="20" spans="1:25" ht="15.75">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -6164,7 +6164,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:25" ht="15.4">
+    <row r="21" spans="1:25" ht="15.75">
       <c r="A21" t="s">
         <v>30</v>
       </c>
@@ -6241,7 +6241,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:25" ht="15.4">
+    <row r="22" spans="1:25" ht="15.75">
       <c r="A22" t="s">
         <v>36</v>
       </c>
@@ -6318,7 +6318,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:25" ht="15.4">
+    <row r="23" spans="1:25" ht="15.75">
       <c r="A23" t="s">
         <v>40</v>
       </c>
@@ -6395,7 +6395,7 @@
         <v>-16</v>
       </c>
     </row>
-    <row r="24" spans="1:25" ht="15.4">
+    <row r="24" spans="1:25" ht="15.75">
       <c r="A24" t="s">
         <v>34</v>
       </c>
@@ -6442,7 +6442,7 @@
         <v>-20</v>
       </c>
     </row>
-    <row r="25" spans="1:25" ht="15.4">
+    <row r="25" spans="1:25" ht="15.75">
       <c r="A25" t="s">
         <v>41</v>
       </c>
@@ -6499,7 +6499,7 @@
       <c r="X25" s="1"/>
       <c r="Y25" s="1"/>
     </row>
-    <row r="26" spans="1:25" ht="15.4">
+    <row r="26" spans="1:25" ht="15.75">
       <c r="A26" t="s">
         <v>26</v>
       </c>
@@ -6587,9 +6587,9 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:Y22"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25">
@@ -6666,7 +6666,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="15.4">
+    <row r="2" spans="1:25" ht="15.75">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -6743,7 +6743,7 @@
         <v>30.3</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15.4">
+    <row r="3" spans="1:25" ht="15.75">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -6820,7 +6820,7 @@
         <v>30.1</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.4">
+    <row r="4" spans="1:25" ht="15.75">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -6897,7 +6897,7 @@
         <v>25.1</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="15.4">
+    <row r="5" spans="1:25" ht="15.75">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -6974,7 +6974,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.4">
+    <row r="6" spans="1:25" ht="15.75">
       <c r="A6" t="s">
         <v>22</v>
       </c>
@@ -7051,7 +7051,7 @@
         <v>21.9</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="15.4">
+    <row r="7" spans="1:25" ht="15.75">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -7128,7 +7128,7 @@
         <v>23.7</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15.4">
+    <row r="8" spans="1:25" ht="15.75">
       <c r="A8" t="s">
         <v>31</v>
       </c>
@@ -7205,7 +7205,7 @@
         <v>5.9</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.4">
+    <row r="9" spans="1:25" ht="15.75">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -7282,7 +7282,7 @@
         <v>18.100000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="15.4">
+    <row r="10" spans="1:25" ht="15.75">
       <c r="A10" t="s">
         <v>36</v>
       </c>
@@ -7359,7 +7359,7 @@
         <v>11.4</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="15.4">
+    <row r="11" spans="1:25" ht="15.75">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -7436,7 +7436,7 @@
         <v>12.6</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="15.4">
+    <row r="12" spans="1:25" ht="15.75">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -7513,7 +7513,7 @@
         <v>6.7</v>
       </c>
     </row>
-    <row r="13" spans="1:25" ht="15.4">
+    <row r="13" spans="1:25" ht="15.75">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -7590,7 +7590,7 @@
         <v>7.7</v>
       </c>
     </row>
-    <row r="14" spans="1:25" ht="15.4">
+    <row r="14" spans="1:25" ht="15.75">
       <c r="A14" t="s">
         <v>29</v>
       </c>
@@ -7667,7 +7667,7 @@
         <v>7.9</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="15.4">
+    <row r="15" spans="1:25" ht="15.75">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -7744,7 +7744,7 @@
         <v>9.3000000000000007</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="15.4">
+    <row r="16" spans="1:25" ht="15.75">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -7821,7 +7821,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:25" ht="15.4">
+    <row r="17" spans="1:25" ht="15.75">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -7898,7 +7898,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="18" spans="1:25" ht="15.4">
+    <row r="18" spans="1:25" ht="15.75">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -7975,7 +7975,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="19" spans="1:25" ht="15.4">
+    <row r="19" spans="1:25" ht="15.75">
       <c r="A19" t="s">
         <v>38</v>
       </c>
@@ -8016,7 +8016,7 @@
       <c r="X19" s="1"/>
       <c r="Y19" s="1"/>
     </row>
-    <row r="20" spans="1:25" ht="15.4">
+    <row r="20" spans="1:25" ht="15.75">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -8093,7 +8093,7 @@
         <v>6.9</v>
       </c>
     </row>
-    <row r="21" spans="1:25" ht="15.4">
+    <row r="21" spans="1:25" ht="15.75">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -8170,7 +8170,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="22" spans="1:25" ht="15.4">
+    <row r="22" spans="1:25" ht="15.75">
       <c r="A22" t="s">
         <v>34</v>
       </c>
@@ -8246,9 +8246,9 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:Y22"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25">
@@ -9904,13 +9904,13 @@
   <sheetPr>
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.1328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="B1">
         <v>1</v>
       </c>
@@ -9923,8 +9923,11 @@
       <c r="E1">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -9940,8 +9943,11 @@
       <c r="E2">
         <v>28.2</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="F2">
+        <v>28.3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -9957,8 +9963,11 @@
       <c r="E3">
         <v>28.3</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="F3">
+        <v>28.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -9974,8 +9983,11 @@
       <c r="E4">
         <v>26.5</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
+      <c r="F4">
+        <v>26.4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -9991,8 +10003,11 @@
       <c r="E5">
         <v>24.6</v>
       </c>
-    </row>
-    <row r="6" spans="1:5">
+      <c r="F5">
+        <v>24.7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -10008,8 +10023,11 @@
       <c r="E6">
         <v>24.1</v>
       </c>
-    </row>
-    <row r="7" spans="1:5">
+      <c r="F6">
+        <v>24.4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -10025,8 +10043,11 @@
       <c r="E7">
         <v>23.7</v>
       </c>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="F7">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -10042,8 +10063,11 @@
       <c r="E8">
         <v>23.2</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
+      <c r="F8">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -10059,8 +10083,11 @@
       <c r="E9">
         <v>13.3</v>
       </c>
-    </row>
-    <row r="10" spans="1:5">
+      <c r="F9">
+        <v>12.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -10076,8 +10103,11 @@
       <c r="E10">
         <v>13</v>
       </c>
-    </row>
-    <row r="11" spans="1:5">
+      <c r="F10">
+        <v>12.8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -10093,8 +10123,11 @@
       <c r="E11">
         <v>12.4</v>
       </c>
-    </row>
-    <row r="12" spans="1:5">
+      <c r="F11">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>26</v>
       </c>
@@ -10110,8 +10143,11 @@
       <c r="E12">
         <v>10.199999999999999</v>
       </c>
-    </row>
-    <row r="13" spans="1:5">
+      <c r="F12">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -10127,8 +10163,11 @@
       <c r="E13">
         <v>8.1999999999999993</v>
       </c>
-    </row>
-    <row r="14" spans="1:5">
+      <c r="F13">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -10144,8 +10183,11 @@
       <c r="E14">
         <v>6.2</v>
       </c>
-    </row>
-    <row r="15" spans="1:5">
+      <c r="F14">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -10161,8 +10203,11 @@
       <c r="E15">
         <v>9.1999999999999993</v>
       </c>
-    </row>
-    <row r="16" spans="1:5">
+      <c r="F15">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -10178,8 +10223,11 @@
       <c r="E16">
         <v>9.1</v>
       </c>
-    </row>
-    <row r="17" spans="1:5">
+      <c r="F16">
+        <v>9.6999999999999993</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -10195,8 +10243,11 @@
       <c r="E17">
         <v>5</v>
       </c>
-    </row>
-    <row r="18" spans="1:5">
+      <c r="F17">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -10212,8 +10263,11 @@
       <c r="E18">
         <v>7.5</v>
       </c>
-    </row>
-    <row r="19" spans="1:5">
+      <c r="F18">
+        <v>8.1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -10229,8 +10283,11 @@
       <c r="E19">
         <v>5.8</v>
       </c>
-    </row>
-    <row r="20" spans="1:5">
+      <c r="F19">
+        <v>5.2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
         <v>33</v>
       </c>
@@ -10246,8 +10303,11 @@
       <c r="E20">
         <v>7.6</v>
       </c>
-    </row>
-    <row r="21" spans="1:5">
+      <c r="F20">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -10263,8 +10323,11 @@
       <c r="E21">
         <v>7.6</v>
       </c>
-    </row>
-    <row r="22" spans="1:5">
+      <c r="F21">
+        <v>8.1999999999999993</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -10280,8 +10343,11 @@
       <c r="E22">
         <v>7</v>
       </c>
-    </row>
-    <row r="23" spans="1:5">
+      <c r="F22">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
       <c r="A23" t="s">
         <v>40</v>
       </c>
@@ -10296,6 +10362,9 @@
       </c>
       <c r="E23">
         <v>4.0999999999999996</v>
+      </c>
+      <c r="F23">
+        <v>3.9</v>
       </c>
     </row>
   </sheetData>
@@ -10308,13 +10377,13 @@
   <sheetPr>
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="B1">
         <v>1</v>
       </c>
@@ -10324,8 +10393,11 @@
       <c r="D1">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -10338,8 +10410,11 @@
       <c r="D2">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="E2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -10352,8 +10427,11 @@
       <c r="D3">
         <v>27</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="E3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -10366,8 +10444,11 @@
       <c r="D4">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="E4">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -10380,8 +10461,11 @@
       <c r="D5">
         <v>43</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="E5">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -10394,8 +10478,11 @@
       <c r="D6">
         <v>50</v>
       </c>
-    </row>
-    <row r="7" spans="1:4">
+      <c r="E6">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -10408,8 +10495,11 @@
       <c r="D7">
         <v>31</v>
       </c>
-    </row>
-    <row r="8" spans="1:4">
+      <c r="E7">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -10422,8 +10512,11 @@
       <c r="D8">
         <v>19</v>
       </c>
-    </row>
-    <row r="9" spans="1:4">
+      <c r="E8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -10436,8 +10529,11 @@
       <c r="D9">
         <v>5</v>
       </c>
-    </row>
-    <row r="10" spans="1:4">
+      <c r="E9">
+        <v>-16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -10450,8 +10546,11 @@
       <c r="D10">
         <v>14</v>
       </c>
-    </row>
-    <row r="11" spans="1:4">
+      <c r="E10">
+        <v>-8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -10464,8 +10563,11 @@
       <c r="D11">
         <v>4</v>
       </c>
-    </row>
-    <row r="12" spans="1:4">
+      <c r="E11">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
       <c r="A12" t="s">
         <v>26</v>
       </c>
@@ -10478,8 +10580,11 @@
       <c r="D12">
         <v>-1</v>
       </c>
-    </row>
-    <row r="13" spans="1:4">
+      <c r="E12">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
       <c r="A13" t="s">
         <v>37</v>
       </c>
@@ -10492,8 +10597,11 @@
       <c r="D13">
         <v>4</v>
       </c>
-    </row>
-    <row r="14" spans="1:4">
+      <c r="E13">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -10506,8 +10614,11 @@
       <c r="D14">
         <v>-17</v>
       </c>
-    </row>
-    <row r="15" spans="1:4">
+      <c r="E14">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -10520,8 +10631,11 @@
       <c r="D15">
         <v>-14</v>
       </c>
-    </row>
-    <row r="16" spans="1:4">
+      <c r="E15">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -10534,8 +10648,11 @@
       <c r="D16">
         <v>9</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="E16">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -10548,8 +10665,11 @@
       <c r="D17">
         <v>10</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
+      <c r="E17">
+        <v>-29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -10562,8 +10682,11 @@
       <c r="D18">
         <v>10</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
+      <c r="E18">
+        <v>-12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -10576,8 +10699,11 @@
       <c r="D19">
         <v>3</v>
       </c>
-    </row>
-    <row r="20" spans="1:4">
+      <c r="E19">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
       <c r="A20" t="s">
         <v>33</v>
       </c>
@@ -10590,8 +10716,11 @@
       <c r="D20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:4">
+      <c r="E20">
+        <v>-4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -10604,8 +10733,11 @@
       <c r="D21">
         <v>4</v>
       </c>
-    </row>
-    <row r="22" spans="1:4">
+      <c r="E21">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
       <c r="A22" t="s">
         <v>35</v>
       </c>
@@ -10618,8 +10750,11 @@
       <c r="D22">
         <v>4</v>
       </c>
-    </row>
-    <row r="23" spans="1:4">
+      <c r="E22">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
       <c r="A23" t="s">
         <v>40</v>
       </c>
@@ -10631,6 +10766,9 @@
       </c>
       <c r="D23">
         <v>2</v>
+      </c>
+      <c r="E23">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -10641,7 +10779,7 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{008844FF-9942-4BA0-9033-82ED2D862880}">
   <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" t="s">
@@ -10920,9 +11058,9 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:Y11"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25">
@@ -10999,7 +11137,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="15.4">
+    <row r="2" spans="1:25" ht="15.75">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -11076,7 +11214,7 @@
         <v>29.7</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15.4">
+    <row r="3" spans="1:25" ht="15.75">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -11153,7 +11291,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.4">
+    <row r="4" spans="1:25" ht="15.75">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -11230,7 +11368,7 @@
         <v>25.3</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="15.4">
+    <row r="5" spans="1:25" ht="15.75">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -11307,7 +11445,7 @@
         <v>25.1</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.4">
+    <row r="6" spans="1:25" ht="15.75">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -11384,7 +11522,7 @@
         <v>14.4</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="15.4">
+    <row r="7" spans="1:25" ht="15.75">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -11461,7 +11599,7 @@
         <v>12.9</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15.4">
+    <row r="8" spans="1:25" ht="15.75">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -11538,7 +11676,7 @@
         <v>12.1</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.4">
+    <row r="9" spans="1:25" ht="15.75">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -11615,7 +11753,7 @@
         <v>12.2</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="15.4">
+    <row r="10" spans="1:25" ht="15.75">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -11692,7 +11830,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="15.4">
+    <row r="11" spans="1:25" ht="15.75">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -11780,7 +11918,7 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:Y11"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
       <c r="B1">
@@ -11856,7 +11994,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="15.4">
+    <row r="2" spans="1:25" ht="15.75">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -11933,7 +12071,7 @@
         <v>36.1</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15.4">
+    <row r="3" spans="1:25" ht="15.75">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -12010,7 +12148,7 @@
         <v>31.8</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.4">
+    <row r="4" spans="1:25" ht="15.75">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -12087,7 +12225,7 @@
         <v>31.1</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="15.4">
+    <row r="5" spans="1:25" ht="15.75">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -12164,7 +12302,7 @@
         <v>28.4</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.4">
+    <row r="6" spans="1:25" ht="15.75">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -12241,7 +12379,7 @@
         <v>19.5</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="15.4">
+    <row r="7" spans="1:25" ht="15.75">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -12318,7 +12456,7 @@
         <v>16.2</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15.4">
+    <row r="8" spans="1:25" ht="15.75">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -12395,7 +12533,7 @@
         <v>15.6</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.4">
+    <row r="9" spans="1:25" ht="15.75">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -12472,7 +12610,7 @@
         <v>10.3</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="15.4">
+    <row r="10" spans="1:25" ht="15.75">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -12549,7 +12687,7 @@
         <v>10.1</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="15.4">
+    <row r="11" spans="1:25" ht="15.75">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -12637,7 +12775,7 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:E12"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="B1">
@@ -12851,7 +12989,7 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="V1:AR11"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="22:44">
       <c r="W1">
@@ -12921,7 +13059,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="22:44" ht="15.4">
+    <row r="2" spans="22:44" ht="15.75">
       <c r="V2" t="s">
         <v>0</v>
       </c>
@@ -12992,7 +13130,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="22:44" ht="15.4">
+    <row r="3" spans="22:44" ht="15.75">
       <c r="V3" t="s">
         <v>2</v>
       </c>
@@ -13063,7 +13201,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="22:44" ht="15.4">
+    <row r="4" spans="22:44" ht="15.75">
       <c r="V4" t="s">
         <v>3</v>
       </c>
@@ -13134,7 +13272,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="22:44" ht="15.4">
+    <row r="5" spans="22:44" ht="15.75">
       <c r="V5" t="s">
         <v>4</v>
       </c>
@@ -13205,7 +13343,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="22:44" ht="15.4">
+    <row r="6" spans="22:44" ht="15.75">
       <c r="V6" t="s">
         <v>1</v>
       </c>
@@ -13276,7 +13414,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="22:44" ht="15.4">
+    <row r="7" spans="22:44" ht="15.75">
       <c r="V7" t="s">
         <v>5</v>
       </c>
@@ -13347,7 +13485,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="22:44" ht="15.4">
+    <row r="8" spans="22:44" ht="15.75">
       <c r="V8" t="s">
         <v>6</v>
       </c>
@@ -13418,7 +13556,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="22:44" ht="15.4">
+    <row r="9" spans="22:44" ht="15.75">
       <c r="V9" t="s">
         <v>7</v>
       </c>
@@ -13489,7 +13627,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="22:44" ht="15.4">
+    <row r="10" spans="22:44" ht="15.75">
       <c r="V10" t="s">
         <v>9</v>
       </c>
@@ -13560,7 +13698,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="22:44" ht="15.4">
+    <row r="11" spans="22:44" ht="15.75">
       <c r="V11" t="s">
         <v>8</v>
       </c>
@@ -13642,7 +13780,7 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:Y11"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
       <c r="B1">
@@ -13718,7 +13856,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="15.4">
+    <row r="2" spans="1:25" ht="15.75">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -13795,7 +13933,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="15.4">
+    <row r="3" spans="1:25" ht="15.75">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -13872,7 +14010,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.4">
+    <row r="4" spans="1:25" ht="15.75">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -13949,7 +14087,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="15.4">
+    <row r="5" spans="1:25" ht="15.75">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -14026,7 +14164,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="15.4">
+    <row r="6" spans="1:25" ht="15.75">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -14103,7 +14241,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="15.4">
+    <row r="7" spans="1:25" ht="15.75">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -14180,7 +14318,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="15.4">
+    <row r="8" spans="1:25" ht="15.75">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -14257,7 +14395,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="15.4">
+    <row r="9" spans="1:25" ht="15.75">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -14334,7 +14472,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="15.4">
+    <row r="10" spans="1:25" ht="15.75">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -14411,7 +14549,7 @@
         <v>-3</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="15.4">
+    <row r="11" spans="1:25" ht="15.75">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -14499,7 +14637,7 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="BR1:CP11"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="70:94">
       <c r="BS1">
@@ -15356,9 +15494,9 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.73046875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -15537,9 +15675,9 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:W23"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="18.75" customHeight="1">
@@ -15610,7 +15748,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="15.4">
+    <row r="2" spans="1:23" ht="15.75">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -15681,7 +15819,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="15.4">
+    <row r="3" spans="1:23" ht="15.75">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -15752,7 +15890,7 @@
         <v>25.3</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="15.4">
+    <row r="4" spans="1:23" ht="15.75">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -15823,7 +15961,7 @@
         <v>23.5</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="15.4">
+    <row r="5" spans="1:23" ht="15.75">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -15894,7 +16032,7 @@
         <v>20.8</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="15.4">
+    <row r="6" spans="1:23" ht="15.75">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -15965,7 +16103,7 @@
         <v>20.2</v>
       </c>
     </row>
-    <row r="7" spans="1:23" ht="15.4">
+    <row r="7" spans="1:23" ht="15.75">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -16036,7 +16174,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="15.4">
+    <row r="8" spans="1:23" ht="15.75">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -16107,7 +16245,7 @@
         <v>19.8</v>
       </c>
     </row>
-    <row r="9" spans="1:23" ht="15.4">
+    <row r="9" spans="1:23" ht="15.75">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -16178,7 +16316,7 @@
         <v>15.8</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="15.4">
+    <row r="10" spans="1:23" ht="15.75">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -16249,7 +16387,7 @@
         <v>13.5</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="15.4">
+    <row r="11" spans="1:23" ht="15.75">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -16320,7 +16458,7 @@
         <v>14.5</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="15.4">
+    <row r="12" spans="1:23" ht="15.75">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -16391,7 +16529,7 @@
         <v>15.4</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="15.4">
+    <row r="13" spans="1:23" ht="15.75">
       <c r="A13" t="s">
         <v>27</v>
       </c>
@@ -16462,7 +16600,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="15.4">
+    <row r="14" spans="1:23" ht="15.75">
       <c r="A14" t="s">
         <v>40</v>
       </c>
@@ -16533,7 +16671,7 @@
         <v>9.6</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="15.4">
+    <row r="15" spans="1:23" ht="15.75">
       <c r="A15" t="s">
         <v>26</v>
       </c>
@@ -16604,7 +16742,7 @@
         <v>11.3</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="15.4">
+    <row r="16" spans="1:23" ht="15.75">
       <c r="A16" t="s">
         <v>39</v>
       </c>
@@ -16675,7 +16813,7 @@
         <v>9.6</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="15.4">
+    <row r="17" spans="1:23" ht="15.75">
       <c r="A17" t="s">
         <v>79</v>
       </c>
@@ -16746,7 +16884,7 @@
         <v>7.7</v>
       </c>
     </row>
-    <row r="18" spans="1:23" ht="15.4">
+    <row r="18" spans="1:23" ht="15.75">
       <c r="A18" t="s">
         <v>36</v>
       </c>
@@ -16817,7 +16955,7 @@
         <v>9.4</v>
       </c>
     </row>
-    <row r="19" spans="1:23" ht="15.4">
+    <row r="19" spans="1:23" ht="15.75">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -16854,7 +16992,7 @@
       <c r="V19" s="1"/>
       <c r="W19" s="1"/>
     </row>
-    <row r="20" spans="1:23" ht="15.4">
+    <row r="20" spans="1:23" ht="15.75">
       <c r="A20" t="s">
         <v>42</v>
       </c>
@@ -16895,7 +17033,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="21" spans="1:23" ht="15.4">
+    <row r="21" spans="1:23" ht="15.75">
       <c r="A21" t="s">
         <v>43</v>
       </c>
@@ -16942,7 +17080,7 @@
       <c r="V21" s="1"/>
       <c r="W21" s="1"/>
     </row>
-    <row r="22" spans="1:23" ht="15.4">
+    <row r="22" spans="1:23" ht="15.75">
       <c r="A22" t="s">
         <v>30</v>
       </c>
@@ -17013,7 +17151,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="15.4">
+    <row r="23" spans="1:23" ht="15.75">
       <c r="A23" t="s">
         <v>41</v>
       </c>

</xml_diff>

<commit_message>
constructor feature tables created
</commit_message>
<xml_diff>
--- a/data/raw/newHistPointAndPrice.xlsx
+++ b/data/raw/newHistPointAndPrice.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE86E263-1D2E-4458-9534-3A0137ACD6EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D3DB95D-C8CE-4418-8532-9F9FAC556734}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" firstSheet="11" activeTab="15" xr2:uid="{2D04FC15-E09F-4251-B381-E10D89E9EC62}"/>
+    <workbookView xWindow="3060" yWindow="1650" windowWidth="21600" windowHeight="11055" tabRatio="864" xr2:uid="{2D04FC15-E09F-4251-B381-E10D89E9EC62}"/>
   </bookViews>
   <sheets>
     <sheet name="2023ConstructorPrice" sheetId="1" r:id="rId1"/>
@@ -12774,10 +12774,10 @@
   <sheetPr>
     <tabColor theme="5"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="B1">
         <v>1</v>
       </c>
@@ -12788,10 +12788,13 @@
         <v>3</v>
       </c>
       <c r="E1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
+        <v>6</v>
+      </c>
+      <c r="F1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -12807,8 +12810,11 @@
       <c r="E2">
         <v>30.2</v>
       </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="F2">
+        <v>30.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -12824,8 +12830,11 @@
       <c r="E3">
         <v>28.6</v>
       </c>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="F3">
+        <v>28.9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -12841,8 +12850,11 @@
       <c r="E4">
         <v>29.1</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
+      <c r="F4">
+        <v>29.2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -12858,8 +12870,11 @@
       <c r="E5">
         <v>24.2</v>
       </c>
-    </row>
-    <row r="6" spans="1:5">
+      <c r="F5">
+        <v>24.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -12875,8 +12890,11 @@
       <c r="E6">
         <v>14.3</v>
       </c>
-    </row>
-    <row r="7" spans="1:5">
+      <c r="F6">
+        <v>14.9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -12892,8 +12910,11 @@
       <c r="E7">
         <v>13.8</v>
       </c>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="F7">
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -12909,8 +12930,11 @@
       <c r="E8">
         <v>8.5</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
+      <c r="F8">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -12926,8 +12950,11 @@
       <c r="E9">
         <v>9.1999999999999993</v>
       </c>
-    </row>
-    <row r="10" spans="1:5">
+      <c r="F9">
+        <v>9.8000000000000007</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -12943,8 +12970,11 @@
       <c r="E10">
         <v>5.6</v>
       </c>
-    </row>
-    <row r="11" spans="1:5">
+      <c r="F10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -12960,8 +12990,11 @@
       <c r="E11">
         <v>8.1</v>
       </c>
-    </row>
-    <row r="12" spans="1:5">
+      <c r="F11">
+        <v>8.6999999999999993</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -12976,6 +13009,9 @@
       </c>
       <c r="E12">
         <v>5</v>
+      </c>
+      <c r="F12">
+        <v>5.6</v>
       </c>
     </row>
   </sheetData>
@@ -12988,784 +13024,784 @@
   <sheetPr>
     <tabColor theme="5"/>
   </sheetPr>
-  <dimension ref="V1:AR11"/>
+  <dimension ref="A1:W11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="22:44">
+    <row r="1" spans="1:23">
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>7</v>
+      </c>
+      <c r="H1">
+        <v>8</v>
+      </c>
+      <c r="I1">
+        <v>9</v>
+      </c>
+      <c r="J1">
+        <v>10</v>
+      </c>
+      <c r="K1">
+        <v>11</v>
+      </c>
+      <c r="L1">
+        <v>12</v>
+      </c>
+      <c r="M1">
+        <v>13</v>
+      </c>
+      <c r="N1">
+        <v>14</v>
+      </c>
+      <c r="O1">
+        <v>15</v>
+      </c>
+      <c r="P1">
+        <v>16</v>
+      </c>
+      <c r="Q1">
+        <v>17</v>
+      </c>
+      <c r="R1">
+        <v>18</v>
+      </c>
+      <c r="S1">
+        <v>19</v>
+      </c>
+      <c r="T1">
+        <v>20</v>
+      </c>
+      <c r="U1">
+        <v>21</v>
+      </c>
+      <c r="V1">
+        <v>22</v>
+      </c>
       <c r="W1">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" ht="15.75">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1">
+        <v>78</v>
+      </c>
+      <c r="C2" s="1">
+        <v>95</v>
+      </c>
+      <c r="D2" s="1">
+        <v>98</v>
+      </c>
+      <c r="E2" s="1">
+        <v>108</v>
+      </c>
+      <c r="F2" s="1">
+        <v>97</v>
+      </c>
+      <c r="G2" s="1">
+        <v>63</v>
+      </c>
+      <c r="H2" s="1">
+        <v>96</v>
+      </c>
+      <c r="I2" s="1">
+        <v>86</v>
+      </c>
+      <c r="J2" s="1">
+        <v>112</v>
+      </c>
+      <c r="K2" s="1">
+        <v>77</v>
+      </c>
+      <c r="L2" s="1">
+        <v>95</v>
+      </c>
+      <c r="M2" s="1">
+        <v>80</v>
+      </c>
+      <c r="N2" s="1">
+        <v>101</v>
+      </c>
+      <c r="O2" s="1">
+        <v>81</v>
+      </c>
+      <c r="P2" s="1">
+        <v>54</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>46</v>
+      </c>
+      <c r="R2" s="1">
+        <v>64</v>
+      </c>
+      <c r="S2" s="1">
+        <v>95</v>
+      </c>
+      <c r="T2" s="1">
+        <v>45</v>
+      </c>
+      <c r="U2" s="1">
+        <v>105</v>
+      </c>
+      <c r="V2" s="1">
+        <v>84</v>
+      </c>
+      <c r="W2" s="1">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" ht="15.75">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1">
+        <v>45</v>
+      </c>
+      <c r="C3" s="1">
+        <v>44</v>
+      </c>
+      <c r="D3" s="1">
+        <v>32</v>
+      </c>
+      <c r="E3" s="1">
+        <v>49</v>
+      </c>
+      <c r="F3" s="1">
+        <v>57</v>
+      </c>
+      <c r="G3" s="1">
+        <v>54</v>
+      </c>
+      <c r="H3" s="1">
+        <v>65</v>
+      </c>
+      <c r="I3" s="1">
+        <v>21</v>
+      </c>
+      <c r="J3" s="1">
+        <v>70</v>
+      </c>
+      <c r="K3" s="1">
+        <v>53</v>
+      </c>
+      <c r="L3" s="1">
+        <v>52</v>
+      </c>
+      <c r="M3" s="1">
+        <v>70</v>
+      </c>
+      <c r="N3" s="1">
+        <v>40</v>
+      </c>
+      <c r="O3" s="1">
+        <v>44</v>
+      </c>
+      <c r="P3" s="1">
+        <v>47</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>44</v>
+      </c>
+      <c r="R3" s="1">
+        <v>53</v>
+      </c>
+      <c r="S3" s="1">
+        <v>21</v>
+      </c>
+      <c r="T3" s="1">
+        <v>69</v>
+      </c>
+      <c r="U3" s="1">
+        <v>24</v>
+      </c>
+      <c r="V3" s="1">
+        <v>45</v>
+      </c>
+      <c r="W3" s="1">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" ht="15.75">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1">
+        <v>31</v>
+      </c>
+      <c r="C4" s="1">
+        <v>59</v>
+      </c>
+      <c r="D4" s="1">
+        <v>3</v>
+      </c>
+      <c r="E4" s="1">
+        <v>63</v>
+      </c>
+      <c r="F4" s="1">
+        <v>56</v>
+      </c>
+      <c r="G4" s="1">
+        <v>37</v>
+      </c>
+      <c r="H4" s="1">
+        <v>38</v>
+      </c>
+      <c r="I4" s="1">
+        <v>46</v>
+      </c>
+      <c r="J4" s="1">
+        <v>73</v>
+      </c>
+      <c r="K4" s="1">
+        <v>25</v>
+      </c>
+      <c r="L4" s="1">
+        <v>32</v>
+      </c>
+      <c r="M4" s="1">
+        <v>38</v>
+      </c>
+      <c r="N4" s="1">
+        <v>34</v>
+      </c>
+      <c r="O4" s="1">
+        <v>67</v>
+      </c>
+      <c r="P4" s="1">
+        <v>70</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>65</v>
+      </c>
+      <c r="R4" s="1">
+        <v>18</v>
+      </c>
+      <c r="S4" s="1">
+        <v>25</v>
+      </c>
+      <c r="T4" s="1">
+        <v>63</v>
+      </c>
+      <c r="U4" s="1">
+        <v>28</v>
+      </c>
+      <c r="V4" s="1">
+        <v>78</v>
+      </c>
+      <c r="W4" s="1">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" ht="15.75">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1">
+        <v>-16</v>
+      </c>
+      <c r="C5" s="1">
+        <v>14</v>
+      </c>
+      <c r="D5" s="1">
+        <v>36</v>
+      </c>
+      <c r="E5" s="1">
+        <v>23</v>
+      </c>
+      <c r="F5" s="1">
+        <v>8</v>
+      </c>
+      <c r="G5" s="1">
+        <v>15</v>
+      </c>
+      <c r="H5" s="1">
+        <v>11</v>
+      </c>
+      <c r="I5" s="1">
+        <v>15</v>
+      </c>
+      <c r="J5" s="1">
+        <v>54</v>
+      </c>
+      <c r="K5" s="1">
+        <v>68</v>
+      </c>
+      <c r="L5" s="1">
+        <v>62</v>
+      </c>
+      <c r="M5" s="1">
+        <v>18</v>
+      </c>
+      <c r="N5" s="1">
+        <v>56</v>
+      </c>
+      <c r="O5" s="1">
+        <v>44</v>
+      </c>
+      <c r="P5" s="1">
+        <v>64</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>66</v>
+      </c>
+      <c r="R5" s="1">
+        <v>110</v>
+      </c>
+      <c r="S5" s="1">
+        <v>36</v>
+      </c>
+      <c r="T5" s="1">
+        <v>57</v>
+      </c>
+      <c r="U5" s="1">
+        <v>65</v>
+      </c>
+      <c r="V5" s="1">
+        <v>34</v>
+      </c>
+      <c r="W5" s="1">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" ht="15.75">
+      <c r="A6" t="s">
         <v>1</v>
       </c>
-      <c r="X1">
+      <c r="B6" s="1">
+        <v>56</v>
+      </c>
+      <c r="C6" s="1">
+        <v>19</v>
+      </c>
+      <c r="D6" s="1">
+        <v>54</v>
+      </c>
+      <c r="E6" s="1">
+        <v>55</v>
+      </c>
+      <c r="F6" s="1">
+        <v>42</v>
+      </c>
+      <c r="G6" s="1">
+        <v>15</v>
+      </c>
+      <c r="H6" s="1">
+        <v>40</v>
+      </c>
+      <c r="I6" s="1">
+        <v>46</v>
+      </c>
+      <c r="J6" s="1">
+        <v>63</v>
+      </c>
+      <c r="K6" s="1">
+        <v>22</v>
+      </c>
+      <c r="L6" s="1">
+        <v>21</v>
+      </c>
+      <c r="M6" s="1">
+        <v>24</v>
+      </c>
+      <c r="N6" s="1">
+        <v>67</v>
+      </c>
+      <c r="O6" s="1">
+        <v>17</v>
+      </c>
+      <c r="P6" s="1">
+        <v>4</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>7</v>
+      </c>
+      <c r="R6" s="1">
+        <v>47</v>
+      </c>
+      <c r="S6" s="1">
+        <v>0</v>
+      </c>
+      <c r="T6" s="1">
+        <v>-7</v>
+      </c>
+      <c r="U6" s="1">
+        <v>77</v>
+      </c>
+      <c r="V6" s="1">
+        <v>56</v>
+      </c>
+      <c r="W6" s="1">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" ht="15.75">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1">
+        <v>8</v>
+      </c>
+      <c r="C7" s="1">
+        <v>28</v>
+      </c>
+      <c r="D7" s="1">
+        <v>11</v>
+      </c>
+      <c r="E7" s="1">
+        <v>25</v>
+      </c>
+      <c r="F7" s="1">
+        <v>28</v>
+      </c>
+      <c r="G7" s="1">
+        <v>42</v>
+      </c>
+      <c r="H7" s="1">
+        <v>33</v>
+      </c>
+      <c r="I7" s="1">
+        <v>24</v>
+      </c>
+      <c r="J7" s="1">
+        <v>21</v>
+      </c>
+      <c r="K7" s="1">
+        <v>-16</v>
+      </c>
+      <c r="L7" s="1">
+        <v>-35</v>
+      </c>
+      <c r="M7" s="1">
+        <v>43</v>
+      </c>
+      <c r="N7" s="1">
+        <v>66</v>
+      </c>
+      <c r="O7" s="1">
+        <v>-16</v>
+      </c>
+      <c r="P7" s="1">
+        <v>13</v>
+      </c>
+      <c r="Q7" s="1">
+        <v>20</v>
+      </c>
+      <c r="R7" s="1">
+        <v>23</v>
+      </c>
+      <c r="S7" s="1">
+        <v>27</v>
+      </c>
+      <c r="T7" s="1">
+        <v>21</v>
+      </c>
+      <c r="U7" s="1">
+        <v>44</v>
+      </c>
+      <c r="V7" s="1">
+        <v>46</v>
+      </c>
+      <c r="W7" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" ht="15.75">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="1">
+        <v>17</v>
+      </c>
+      <c r="C8" s="1">
+        <v>15</v>
+      </c>
+      <c r="D8" s="1">
+        <v>13</v>
+      </c>
+      <c r="E8" s="1">
+        <v>-23</v>
+      </c>
+      <c r="F8" s="1">
+        <v>17</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1</v>
+      </c>
+      <c r="H8" s="1">
+        <v>20</v>
+      </c>
+      <c r="I8" s="1">
+        <v>6</v>
+      </c>
+      <c r="J8" s="1">
+        <v>20</v>
+      </c>
+      <c r="K8" s="1">
+        <v>5</v>
+      </c>
+      <c r="L8" s="1">
+        <v>8</v>
+      </c>
+      <c r="M8" s="1">
+        <v>18</v>
+      </c>
+      <c r="N8" s="1">
+        <v>40</v>
+      </c>
+      <c r="O8" s="1">
+        <v>-12</v>
+      </c>
+      <c r="P8" s="1">
+        <v>-4</v>
+      </c>
+      <c r="Q8" s="1">
+        <v>15</v>
+      </c>
+      <c r="R8" s="1">
+        <v>-4</v>
+      </c>
+      <c r="S8" s="1">
+        <v>34</v>
+      </c>
+      <c r="T8" s="1">
+        <v>42</v>
+      </c>
+      <c r="U8" s="1">
+        <v>31</v>
+      </c>
+      <c r="V8" s="1">
+        <v>26</v>
+      </c>
+      <c r="W8" s="1">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" ht="15.75">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" s="1">
+        <v>31</v>
+      </c>
+      <c r="C9" s="1">
+        <v>7</v>
+      </c>
+      <c r="D9" s="1">
+        <v>26</v>
+      </c>
+      <c r="E9" s="1">
+        <v>-10</v>
+      </c>
+      <c r="F9" s="1">
+        <v>8</v>
+      </c>
+      <c r="G9" s="1">
+        <v>22</v>
+      </c>
+      <c r="H9" s="1">
+        <v>19</v>
+      </c>
+      <c r="I9" s="1">
+        <v>11</v>
+      </c>
+      <c r="J9" s="1">
+        <v>16</v>
+      </c>
+      <c r="K9" s="1">
+        <v>-5</v>
+      </c>
+      <c r="L9" s="1">
+        <v>6</v>
+      </c>
+      <c r="M9" s="1">
+        <v>26</v>
+      </c>
+      <c r="N9" s="1">
+        <v>4</v>
+      </c>
+      <c r="O9" s="1">
+        <v>12</v>
+      </c>
+      <c r="P9" s="1">
+        <v>-8</v>
+      </c>
+      <c r="Q9" s="1">
+        <v>-10</v>
+      </c>
+      <c r="R9" s="1">
+        <v>39</v>
+      </c>
+      <c r="S9" s="1">
+        <v>15</v>
+      </c>
+      <c r="T9" s="1">
+        <v>14</v>
+      </c>
+      <c r="U9" s="1">
+        <v>-31</v>
+      </c>
+      <c r="V9" s="1">
+        <v>12</v>
+      </c>
+      <c r="W9" s="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" ht="15.75">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1">
+        <v>12</v>
+      </c>
+      <c r="C10" s="1">
+        <v>13</v>
+      </c>
+      <c r="D10" s="1">
+        <v>18</v>
+      </c>
+      <c r="E10" s="1">
+        <v>17</v>
+      </c>
+      <c r="F10" s="1">
+        <v>15</v>
+      </c>
+      <c r="G10" s="1">
+        <v>7</v>
+      </c>
+      <c r="H10" s="1">
+        <v>17</v>
+      </c>
+      <c r="I10" s="1">
+        <v>4</v>
+      </c>
+      <c r="J10" s="1">
+        <v>14</v>
+      </c>
+      <c r="K10" s="1">
+        <v>-18</v>
+      </c>
+      <c r="L10" s="1">
+        <v>10</v>
+      </c>
+      <c r="M10" s="1">
+        <v>23</v>
+      </c>
+      <c r="N10" s="1">
+        <v>26</v>
+      </c>
+      <c r="O10" s="1">
+        <v>0</v>
+      </c>
+      <c r="P10" s="1">
+        <v>18</v>
+      </c>
+      <c r="Q10" s="1">
+        <v>15</v>
+      </c>
+      <c r="R10" s="1">
+        <v>6</v>
+      </c>
+      <c r="S10" s="1">
+        <v>30</v>
+      </c>
+      <c r="T10" s="1">
+        <v>-7</v>
+      </c>
+      <c r="U10" s="1">
+        <v>-19</v>
+      </c>
+      <c r="V10" s="1">
+        <v>12</v>
+      </c>
+      <c r="W10" s="1">
         <v>2</v>
       </c>
-      <c r="Y1">
-        <v>3</v>
-      </c>
-      <c r="Z1">
-        <v>4</v>
-      </c>
-      <c r="AA1">
+    </row>
+    <row r="11" spans="1:23" ht="15.75">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="1">
+        <v>25</v>
+      </c>
+      <c r="C11" s="1">
+        <v>-16</v>
+      </c>
+      <c r="D11" s="1">
+        <v>-5</v>
+      </c>
+      <c r="E11" s="1">
         <v>5</v>
       </c>
-      <c r="AB1">
+      <c r="F11" s="1">
+        <v>1</v>
+      </c>
+      <c r="G11" s="1">
+        <v>1</v>
+      </c>
+      <c r="H11" s="1">
+        <v>5</v>
+      </c>
+      <c r="I11" s="1">
+        <v>-2</v>
+      </c>
+      <c r="J11" s="1">
+        <v>35</v>
+      </c>
+      <c r="K11" s="1">
+        <v>19</v>
+      </c>
+      <c r="L11" s="1">
+        <v>9</v>
+      </c>
+      <c r="M11" s="1">
+        <v>21</v>
+      </c>
+      <c r="N11" s="1">
+        <v>9</v>
+      </c>
+      <c r="O11" s="1">
+        <v>20</v>
+      </c>
+      <c r="P11" s="1">
+        <v>19</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>-35</v>
+      </c>
+      <c r="R11" s="1">
+        <v>-10</v>
+      </c>
+      <c r="S11" s="1">
+        <v>29</v>
+      </c>
+      <c r="T11" s="1">
+        <v>20</v>
+      </c>
+      <c r="U11" s="1">
+        <v>2</v>
+      </c>
+      <c r="V11" s="1">
         <v>7</v>
       </c>
-      <c r="AC1">
-        <v>8</v>
-      </c>
-      <c r="AD1">
-        <v>9</v>
-      </c>
-      <c r="AE1">
-        <v>10</v>
-      </c>
-      <c r="AF1">
-        <v>11</v>
-      </c>
-      <c r="AG1">
-        <v>12</v>
-      </c>
-      <c r="AH1">
-        <v>13</v>
-      </c>
-      <c r="AI1">
-        <v>14</v>
-      </c>
-      <c r="AJ1">
-        <v>15</v>
-      </c>
-      <c r="AK1">
-        <v>16</v>
-      </c>
-      <c r="AL1">
-        <v>17</v>
-      </c>
-      <c r="AM1">
-        <v>18</v>
-      </c>
-      <c r="AN1">
-        <v>19</v>
-      </c>
-      <c r="AO1">
-        <v>20</v>
-      </c>
-      <c r="AP1">
-        <v>21</v>
-      </c>
-      <c r="AQ1">
-        <v>22</v>
-      </c>
-      <c r="AR1">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="22:44" ht="15.75">
-      <c r="V2" t="s">
-        <v>0</v>
-      </c>
-      <c r="W2" s="1">
-        <v>78</v>
-      </c>
-      <c r="X2" s="1">
-        <v>95</v>
-      </c>
-      <c r="Y2" s="1">
-        <v>98</v>
-      </c>
-      <c r="Z2" s="1">
-        <v>108</v>
-      </c>
-      <c r="AA2" s="1">
-        <v>97</v>
-      </c>
-      <c r="AB2" s="1">
-        <v>63</v>
-      </c>
-      <c r="AC2" s="1">
-        <v>96</v>
-      </c>
-      <c r="AD2" s="1">
-        <v>86</v>
-      </c>
-      <c r="AE2" s="1">
-        <v>112</v>
-      </c>
-      <c r="AF2" s="1">
-        <v>77</v>
-      </c>
-      <c r="AG2" s="1">
-        <v>95</v>
-      </c>
-      <c r="AH2" s="1">
-        <v>80</v>
-      </c>
-      <c r="AI2" s="1">
-        <v>101</v>
-      </c>
-      <c r="AJ2" s="1">
-        <v>81</v>
-      </c>
-      <c r="AK2" s="1">
-        <v>54</v>
-      </c>
-      <c r="AL2" s="1">
-        <v>46</v>
-      </c>
-      <c r="AM2" s="1">
-        <v>64</v>
-      </c>
-      <c r="AN2" s="1">
-        <v>95</v>
-      </c>
-      <c r="AO2" s="1">
-        <v>45</v>
-      </c>
-      <c r="AP2" s="1">
-        <v>105</v>
-      </c>
-      <c r="AQ2" s="1">
-        <v>84</v>
-      </c>
-      <c r="AR2" s="1">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="3" spans="22:44" ht="15.75">
-      <c r="V3" t="s">
-        <v>2</v>
-      </c>
-      <c r="W3" s="1">
-        <v>45</v>
-      </c>
-      <c r="X3" s="1">
-        <v>44</v>
-      </c>
-      <c r="Y3" s="1">
-        <v>32</v>
-      </c>
-      <c r="Z3" s="1">
-        <v>49</v>
-      </c>
-      <c r="AA3" s="1">
-        <v>57</v>
-      </c>
-      <c r="AB3" s="1">
-        <v>54</v>
-      </c>
-      <c r="AC3" s="1">
-        <v>65</v>
-      </c>
-      <c r="AD3" s="1">
-        <v>21</v>
-      </c>
-      <c r="AE3" s="1">
-        <v>70</v>
-      </c>
-      <c r="AF3" s="1">
-        <v>53</v>
-      </c>
-      <c r="AG3" s="1">
-        <v>52</v>
-      </c>
-      <c r="AH3" s="1">
-        <v>70</v>
-      </c>
-      <c r="AI3" s="1">
-        <v>40</v>
-      </c>
-      <c r="AJ3" s="1">
-        <v>44</v>
-      </c>
-      <c r="AK3" s="1">
-        <v>47</v>
-      </c>
-      <c r="AL3" s="1">
-        <v>44</v>
-      </c>
-      <c r="AM3" s="1">
-        <v>53</v>
-      </c>
-      <c r="AN3" s="1">
-        <v>21</v>
-      </c>
-      <c r="AO3" s="1">
-        <v>69</v>
-      </c>
-      <c r="AP3" s="1">
-        <v>24</v>
-      </c>
-      <c r="AQ3" s="1">
-        <v>45</v>
-      </c>
-      <c r="AR3" s="1">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="22:44" ht="15.75">
-      <c r="V4" t="s">
-        <v>3</v>
-      </c>
-      <c r="W4" s="1">
-        <v>31</v>
-      </c>
-      <c r="X4" s="1">
-        <v>59</v>
-      </c>
-      <c r="Y4" s="1">
-        <v>3</v>
-      </c>
-      <c r="Z4" s="1">
-        <v>63</v>
-      </c>
-      <c r="AA4" s="1">
-        <v>56</v>
-      </c>
-      <c r="AB4" s="1">
-        <v>37</v>
-      </c>
-      <c r="AC4" s="1">
-        <v>38</v>
-      </c>
-      <c r="AD4" s="1">
-        <v>46</v>
-      </c>
-      <c r="AE4" s="1">
-        <v>73</v>
-      </c>
-      <c r="AF4" s="1">
-        <v>25</v>
-      </c>
-      <c r="AG4" s="1">
-        <v>32</v>
-      </c>
-      <c r="AH4" s="1">
-        <v>38</v>
-      </c>
-      <c r="AI4" s="1">
-        <v>34</v>
-      </c>
-      <c r="AJ4" s="1">
-        <v>67</v>
-      </c>
-      <c r="AK4" s="1">
-        <v>70</v>
-      </c>
-      <c r="AL4" s="1">
-        <v>65</v>
-      </c>
-      <c r="AM4" s="1">
-        <v>18</v>
-      </c>
-      <c r="AN4" s="1">
-        <v>25</v>
-      </c>
-      <c r="AO4" s="1">
-        <v>63</v>
-      </c>
-      <c r="AP4" s="1">
-        <v>28</v>
-      </c>
-      <c r="AQ4" s="1">
-        <v>78</v>
-      </c>
-      <c r="AR4" s="1">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="22:44" ht="15.75">
-      <c r="V5" t="s">
-        <v>4</v>
-      </c>
-      <c r="W5" s="1">
-        <v>-16</v>
-      </c>
-      <c r="X5" s="1">
-        <v>14</v>
-      </c>
-      <c r="Y5" s="1">
-        <v>36</v>
-      </c>
-      <c r="Z5" s="1">
-        <v>23</v>
-      </c>
-      <c r="AA5" s="1">
-        <v>8</v>
-      </c>
-      <c r="AB5" s="1">
-        <v>15</v>
-      </c>
-      <c r="AC5" s="1">
-        <v>11</v>
-      </c>
-      <c r="AD5" s="1">
-        <v>15</v>
-      </c>
-      <c r="AE5" s="1">
-        <v>54</v>
-      </c>
-      <c r="AF5" s="1">
-        <v>68</v>
-      </c>
-      <c r="AG5" s="1">
-        <v>62</v>
-      </c>
-      <c r="AH5" s="1">
-        <v>18</v>
-      </c>
-      <c r="AI5" s="1">
-        <v>56</v>
-      </c>
-      <c r="AJ5" s="1">
-        <v>44</v>
-      </c>
-      <c r="AK5" s="1">
-        <v>64</v>
-      </c>
-      <c r="AL5" s="1">
-        <v>66</v>
-      </c>
-      <c r="AM5" s="1">
-        <v>110</v>
-      </c>
-      <c r="AN5" s="1">
-        <v>36</v>
-      </c>
-      <c r="AO5" s="1">
-        <v>57</v>
-      </c>
-      <c r="AP5" s="1">
-        <v>65</v>
-      </c>
-      <c r="AQ5" s="1">
-        <v>34</v>
-      </c>
-      <c r="AR5" s="1">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="22:44" ht="15.75">
-      <c r="V6" t="s">
-        <v>1</v>
-      </c>
-      <c r="W6" s="1">
-        <v>56</v>
-      </c>
-      <c r="X6" s="1">
-        <v>19</v>
-      </c>
-      <c r="Y6" s="1">
-        <v>54</v>
-      </c>
-      <c r="Z6" s="1">
-        <v>55</v>
-      </c>
-      <c r="AA6" s="1">
-        <v>42</v>
-      </c>
-      <c r="AB6" s="1">
-        <v>15</v>
-      </c>
-      <c r="AC6" s="1">
-        <v>40</v>
-      </c>
-      <c r="AD6" s="1">
-        <v>46</v>
-      </c>
-      <c r="AE6" s="1">
-        <v>63</v>
-      </c>
-      <c r="AF6" s="1">
-        <v>22</v>
-      </c>
-      <c r="AG6" s="1">
-        <v>21</v>
-      </c>
-      <c r="AH6" s="1">
-        <v>24</v>
-      </c>
-      <c r="AI6" s="1">
-        <v>67</v>
-      </c>
-      <c r="AJ6" s="1">
-        <v>17</v>
-      </c>
-      <c r="AK6" s="1">
-        <v>4</v>
-      </c>
-      <c r="AL6" s="1">
-        <v>7</v>
-      </c>
-      <c r="AM6" s="1">
-        <v>47</v>
-      </c>
-      <c r="AN6" s="1">
-        <v>0</v>
-      </c>
-      <c r="AO6" s="1">
-        <v>-7</v>
-      </c>
-      <c r="AP6" s="1">
-        <v>77</v>
-      </c>
-      <c r="AQ6" s="1">
-        <v>56</v>
-      </c>
-      <c r="AR6" s="1">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="22:44" ht="15.75">
-      <c r="V7" t="s">
-        <v>5</v>
-      </c>
-      <c r="W7" s="1">
-        <v>8</v>
-      </c>
-      <c r="X7" s="1">
-        <v>28</v>
-      </c>
-      <c r="Y7" s="1">
-        <v>11</v>
-      </c>
-      <c r="Z7" s="1">
-        <v>25</v>
-      </c>
-      <c r="AA7" s="1">
-        <v>28</v>
-      </c>
-      <c r="AB7" s="1">
-        <v>42</v>
-      </c>
-      <c r="AC7" s="1">
-        <v>33</v>
-      </c>
-      <c r="AD7" s="1">
-        <v>24</v>
-      </c>
-      <c r="AE7" s="1">
-        <v>21</v>
-      </c>
-      <c r="AF7" s="1">
-        <v>-16</v>
-      </c>
-      <c r="AG7" s="1">
-        <v>-35</v>
-      </c>
-      <c r="AH7" s="1">
-        <v>43</v>
-      </c>
-      <c r="AI7" s="1">
-        <v>66</v>
-      </c>
-      <c r="AJ7" s="1">
-        <v>-16</v>
-      </c>
-      <c r="AK7" s="1">
-        <v>13</v>
-      </c>
-      <c r="AL7" s="1">
-        <v>20</v>
-      </c>
-      <c r="AM7" s="1">
-        <v>23</v>
-      </c>
-      <c r="AN7" s="1">
-        <v>27</v>
-      </c>
-      <c r="AO7" s="1">
-        <v>21</v>
-      </c>
-      <c r="AP7" s="1">
-        <v>44</v>
-      </c>
-      <c r="AQ7" s="1">
-        <v>46</v>
-      </c>
-      <c r="AR7" s="1">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="22:44" ht="15.75">
-      <c r="V8" t="s">
-        <v>6</v>
-      </c>
-      <c r="W8" s="1">
-        <v>17</v>
-      </c>
-      <c r="X8" s="1">
-        <v>15</v>
-      </c>
-      <c r="Y8" s="1">
-        <v>13</v>
-      </c>
-      <c r="Z8" s="1">
-        <v>-23</v>
-      </c>
-      <c r="AA8" s="1">
-        <v>17</v>
-      </c>
-      <c r="AB8" s="1">
-        <v>1</v>
-      </c>
-      <c r="AC8" s="1">
-        <v>20</v>
-      </c>
-      <c r="AD8" s="1">
-        <v>6</v>
-      </c>
-      <c r="AE8" s="1">
-        <v>20</v>
-      </c>
-      <c r="AF8" s="1">
-        <v>5</v>
-      </c>
-      <c r="AG8" s="1">
-        <v>8</v>
-      </c>
-      <c r="AH8" s="1">
-        <v>18</v>
-      </c>
-      <c r="AI8" s="1">
-        <v>40</v>
-      </c>
-      <c r="AJ8" s="1">
-        <v>-12</v>
-      </c>
-      <c r="AK8" s="1">
-        <v>-4</v>
-      </c>
-      <c r="AL8" s="1">
-        <v>15</v>
-      </c>
-      <c r="AM8" s="1">
-        <v>-4</v>
-      </c>
-      <c r="AN8" s="1">
-        <v>34</v>
-      </c>
-      <c r="AO8" s="1">
-        <v>42</v>
-      </c>
-      <c r="AP8" s="1">
-        <v>31</v>
-      </c>
-      <c r="AQ8" s="1">
-        <v>26</v>
-      </c>
-      <c r="AR8" s="1">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="22:44" ht="15.75">
-      <c r="V9" t="s">
-        <v>7</v>
-      </c>
-      <c r="W9" s="1">
-        <v>31</v>
-      </c>
-      <c r="X9" s="1">
-        <v>7</v>
-      </c>
-      <c r="Y9" s="1">
-        <v>26</v>
-      </c>
-      <c r="Z9" s="1">
-        <v>-10</v>
-      </c>
-      <c r="AA9" s="1">
-        <v>8</v>
-      </c>
-      <c r="AB9" s="1">
-        <v>22</v>
-      </c>
-      <c r="AC9" s="1">
-        <v>19</v>
-      </c>
-      <c r="AD9" s="1">
-        <v>11</v>
-      </c>
-      <c r="AE9" s="1">
-        <v>16</v>
-      </c>
-      <c r="AF9" s="1">
-        <v>-5</v>
-      </c>
-      <c r="AG9" s="1">
-        <v>6</v>
-      </c>
-      <c r="AH9" s="1">
-        <v>26</v>
-      </c>
-      <c r="AI9" s="1">
-        <v>4</v>
-      </c>
-      <c r="AJ9" s="1">
-        <v>12</v>
-      </c>
-      <c r="AK9" s="1">
-        <v>-8</v>
-      </c>
-      <c r="AL9" s="1">
-        <v>-10</v>
-      </c>
-      <c r="AM9" s="1">
-        <v>39</v>
-      </c>
-      <c r="AN9" s="1">
-        <v>15</v>
-      </c>
-      <c r="AO9" s="1">
-        <v>14</v>
-      </c>
-      <c r="AP9" s="1">
-        <v>-31</v>
-      </c>
-      <c r="AQ9" s="1">
-        <v>12</v>
-      </c>
-      <c r="AR9" s="1">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="22:44" ht="15.75">
-      <c r="V10" t="s">
-        <v>9</v>
-      </c>
-      <c r="W10" s="1">
-        <v>12</v>
-      </c>
-      <c r="X10" s="1">
-        <v>13</v>
-      </c>
-      <c r="Y10" s="1">
-        <v>18</v>
-      </c>
-      <c r="Z10" s="1">
-        <v>17</v>
-      </c>
-      <c r="AA10" s="1">
-        <v>15</v>
-      </c>
-      <c r="AB10" s="1">
-        <v>7</v>
-      </c>
-      <c r="AC10" s="1">
-        <v>17</v>
-      </c>
-      <c r="AD10" s="1">
-        <v>4</v>
-      </c>
-      <c r="AE10" s="1">
-        <v>14</v>
-      </c>
-      <c r="AF10" s="1">
-        <v>-18</v>
-      </c>
-      <c r="AG10" s="1">
-        <v>10</v>
-      </c>
-      <c r="AH10" s="1">
-        <v>23</v>
-      </c>
-      <c r="AI10" s="1">
-        <v>26</v>
-      </c>
-      <c r="AJ10" s="1">
-        <v>0</v>
-      </c>
-      <c r="AK10" s="1">
-        <v>18</v>
-      </c>
-      <c r="AL10" s="1">
-        <v>15</v>
-      </c>
-      <c r="AM10" s="1">
-        <v>6</v>
-      </c>
-      <c r="AN10" s="1">
-        <v>30</v>
-      </c>
-      <c r="AO10" s="1">
-        <v>-7</v>
-      </c>
-      <c r="AP10" s="1">
-        <v>-19</v>
-      </c>
-      <c r="AQ10" s="1">
-        <v>12</v>
-      </c>
-      <c r="AR10" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="22:44" ht="15.75">
-      <c r="V11" t="s">
-        <v>8</v>
-      </c>
       <c r="W11" s="1">
-        <v>25</v>
-      </c>
-      <c r="X11" s="1">
-        <v>-16</v>
-      </c>
-      <c r="Y11" s="1">
-        <v>-5</v>
-      </c>
-      <c r="Z11" s="1">
-        <v>5</v>
-      </c>
-      <c r="AA11" s="1">
-        <v>1</v>
-      </c>
-      <c r="AB11" s="1">
-        <v>1</v>
-      </c>
-      <c r="AC11" s="1">
-        <v>5</v>
-      </c>
-      <c r="AD11" s="1">
-        <v>-2</v>
-      </c>
-      <c r="AE11" s="1">
-        <v>35</v>
-      </c>
-      <c r="AF11" s="1">
-        <v>19</v>
-      </c>
-      <c r="AG11" s="1">
-        <v>9</v>
-      </c>
-      <c r="AH11" s="1">
-        <v>21</v>
-      </c>
-      <c r="AI11" s="1">
-        <v>9</v>
-      </c>
-      <c r="AJ11" s="1">
-        <v>20</v>
-      </c>
-      <c r="AK11" s="1">
-        <v>19</v>
-      </c>
-      <c r="AL11" s="1">
-        <v>-35</v>
-      </c>
-      <c r="AM11" s="1">
-        <v>-10</v>
-      </c>
-      <c r="AN11" s="1">
-        <v>29</v>
-      </c>
-      <c r="AO11" s="1">
-        <v>20</v>
-      </c>
-      <c r="AP11" s="1">
-        <v>2</v>
-      </c>
-      <c r="AQ11" s="1">
-        <v>7</v>
-      </c>
-      <c r="AR11" s="1">
         <v>12</v>
       </c>
     </row>
@@ -14636,850 +14672,850 @@
   <sheetPr>
     <tabColor theme="5"/>
   </sheetPr>
-  <dimension ref="BR1:CP11"/>
+  <dimension ref="A1:Y11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="70:94">
-      <c r="BS1">
+    <row r="1" spans="1:25">
+      <c r="B1">
         <v>1</v>
       </c>
-      <c r="BT1">
+      <c r="C1">
         <v>2</v>
       </c>
-      <c r="BU1">
+      <c r="D1">
         <v>3</v>
       </c>
-      <c r="BV1">
+      <c r="E1">
         <v>4</v>
       </c>
-      <c r="BW1">
+      <c r="F1">
         <v>5</v>
       </c>
-      <c r="BX1">
+      <c r="G1">
         <v>6</v>
       </c>
-      <c r="BY1">
+      <c r="H1">
         <v>7</v>
       </c>
-      <c r="BZ1">
+      <c r="I1">
         <v>8</v>
       </c>
-      <c r="CA1">
+      <c r="J1">
         <v>9</v>
       </c>
-      <c r="CB1">
+      <c r="K1">
         <v>10</v>
       </c>
-      <c r="CC1">
+      <c r="L1">
         <v>11</v>
       </c>
-      <c r="CD1">
+      <c r="M1">
         <v>12</v>
       </c>
-      <c r="CE1">
+      <c r="N1">
         <v>13</v>
       </c>
-      <c r="CF1">
+      <c r="O1">
         <v>14</v>
       </c>
-      <c r="CG1">
+      <c r="P1">
         <v>15</v>
       </c>
-      <c r="CH1">
+      <c r="Q1">
         <v>16</v>
       </c>
-      <c r="CI1">
+      <c r="R1">
         <v>17</v>
       </c>
-      <c r="CJ1">
+      <c r="S1">
         <v>18</v>
       </c>
-      <c r="CK1">
+      <c r="T1">
         <v>19</v>
       </c>
-      <c r="CL1">
+      <c r="U1">
         <v>20</v>
       </c>
-      <c r="CM1">
+      <c r="V1">
         <v>21</v>
       </c>
-      <c r="CN1">
+      <c r="W1">
         <v>22</v>
       </c>
-      <c r="CO1">
+      <c r="X1">
         <v>23</v>
       </c>
-      <c r="CP1">
+      <c r="Y1">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="70:94">
-      <c r="BR2" t="s">
+    <row r="2" spans="1:25">
+      <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="BS2" s="2">
+      <c r="B2" s="2">
         <v>71</v>
       </c>
-      <c r="BT2" s="2">
+      <c r="C2" s="2">
         <v>101</v>
       </c>
-      <c r="BU2" s="2">
+      <c r="D2" s="2">
         <v>71</v>
       </c>
-      <c r="BV2" s="2">
+      <c r="E2" s="2">
         <v>92</v>
       </c>
-      <c r="BW2" s="2">
+      <c r="F2" s="2">
         <v>86</v>
       </c>
-      <c r="BX2" s="2">
+      <c r="G2" s="2">
         <v>118</v>
       </c>
-      <c r="BY2" s="2">
+      <c r="H2" s="2">
         <v>82</v>
       </c>
-      <c r="BZ2" s="2">
+      <c r="I2" s="2">
         <v>83</v>
       </c>
-      <c r="CA2" s="2">
+      <c r="J2" s="2">
         <v>88</v>
       </c>
-      <c r="CB2" s="2">
+      <c r="K2" s="2">
         <v>40</v>
       </c>
-      <c r="CC2" s="2">
+      <c r="L2" s="2">
         <v>100</v>
       </c>
-      <c r="CD2" s="2">
+      <c r="M2" s="2">
         <v>90</v>
       </c>
-      <c r="CE2" s="2">
+      <c r="N2" s="2">
         <v>93</v>
       </c>
-      <c r="CF2" s="2">
+      <c r="O2" s="2">
         <v>100</v>
       </c>
-      <c r="CG2" s="2">
+      <c r="P2" s="2">
         <v>52</v>
       </c>
-      <c r="CH2" s="2">
+      <c r="Q2" s="2">
         <v>97</v>
       </c>
-      <c r="CI2" s="2">
+      <c r="R2" s="2">
         <v>6</v>
       </c>
-      <c r="CJ2" s="2">
+      <c r="S2" s="2">
         <v>64</v>
       </c>
-      <c r="CK2" s="2">
+      <c r="T2" s="2">
         <v>22</v>
       </c>
-      <c r="CL2" s="2">
+      <c r="U2" s="2">
         <v>86</v>
       </c>
-      <c r="CM2" s="2">
+      <c r="V2" s="2">
         <v>63</v>
       </c>
-      <c r="CN2" s="2">
+      <c r="W2" s="2">
         <v>-34</v>
       </c>
-      <c r="CO2" s="2">
+      <c r="X2" s="2">
         <v>96</v>
       </c>
-      <c r="CP2" s="2">
+      <c r="Y2" s="2">
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="70:94">
-      <c r="BR3" t="s">
+    <row r="3" spans="1:25">
+      <c r="A3" t="s">
         <v>0</v>
       </c>
-      <c r="BS3" s="2">
+      <c r="B3" s="2">
         <v>19</v>
       </c>
-      <c r="BT3" s="2">
+      <c r="C3" s="2">
         <v>67</v>
       </c>
-      <c r="BU3" s="2">
+      <c r="D3" s="2">
         <v>46</v>
       </c>
-      <c r="BV3" s="2">
+      <c r="E3" s="2">
         <v>46</v>
       </c>
-      <c r="BW3" s="2">
+      <c r="F3" s="2">
         <v>21</v>
       </c>
-      <c r="BX3" s="2">
+      <c r="G3" s="2">
         <v>60</v>
       </c>
-      <c r="BY3" s="2">
+      <c r="H3" s="2">
         <v>71</v>
       </c>
-      <c r="BZ3" s="2">
+      <c r="I3" s="2">
         <v>23</v>
       </c>
-      <c r="CA3" s="2">
+      <c r="J3" s="2">
         <v>28</v>
       </c>
-      <c r="CB3" s="2">
+      <c r="K3" s="2">
         <v>51</v>
       </c>
-      <c r="CC3" s="2">
+      <c r="L3" s="2">
         <v>1</v>
       </c>
-      <c r="CD3" s="2">
+      <c r="M3" s="2">
         <v>41</v>
       </c>
-      <c r="CE3" s="2">
+      <c r="N3" s="2">
         <v>55</v>
       </c>
-      <c r="CF3" s="2">
+      <c r="O3" s="2">
         <v>39</v>
       </c>
-      <c r="CG3" s="2">
+      <c r="P3" s="2">
         <v>47</v>
       </c>
-      <c r="CH3" s="2">
+      <c r="Q3" s="2">
         <v>56</v>
       </c>
-      <c r="CI3" s="2">
+      <c r="R3" s="2">
         <v>85</v>
       </c>
-      <c r="CJ3" s="2">
+      <c r="S3" s="2">
         <v>51</v>
       </c>
-      <c r="CK3" s="2">
+      <c r="T3" s="2">
         <v>92</v>
       </c>
-      <c r="CL3" s="2">
+      <c r="U3" s="2">
         <v>36</v>
       </c>
-      <c r="CM3" s="2">
+      <c r="V3" s="2">
         <v>88</v>
       </c>
-      <c r="CN3" s="2">
+      <c r="W3" s="2">
         <v>85</v>
       </c>
-      <c r="CO3" s="2">
+      <c r="X3" s="2">
         <v>67</v>
       </c>
-      <c r="CP3" s="2">
+      <c r="Y3" s="2">
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="70:94">
-      <c r="BR4" t="s">
+    <row r="4" spans="1:25">
+      <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="BS4" s="2">
+      <c r="B4" s="2">
         <v>67</v>
       </c>
-      <c r="BT4" s="2">
+      <c r="C4" s="2">
         <v>69</v>
       </c>
-      <c r="BU4" s="2">
+      <c r="D4" s="2">
         <v>56</v>
       </c>
-      <c r="BV4" s="2">
+      <c r="E4" s="2">
         <v>60</v>
       </c>
-      <c r="BW4" s="2">
+      <c r="F4" s="2">
         <v>46</v>
       </c>
-      <c r="BX4" s="2">
+      <c r="G4" s="2">
         <v>51</v>
       </c>
-      <c r="BY4" s="2">
+      <c r="H4" s="2">
         <v>6</v>
       </c>
-      <c r="BZ4" s="2">
+      <c r="I4" s="2">
         <v>9</v>
       </c>
-      <c r="CA4" s="2">
+      <c r="J4" s="2">
         <v>24</v>
       </c>
-      <c r="CB4" s="2">
+      <c r="K4" s="2">
         <v>87</v>
       </c>
-      <c r="CC4" s="2">
+      <c r="L4" s="2">
         <v>19</v>
       </c>
-      <c r="CD4" s="2">
+      <c r="M4" s="2">
         <v>7</v>
       </c>
-      <c r="CE4" s="2">
+      <c r="N4" s="2">
         <v>50</v>
       </c>
-      <c r="CF4" s="2">
+      <c r="O4" s="2">
         <v>54</v>
       </c>
-      <c r="CG4" s="2">
+      <c r="P4" s="2">
         <v>30</v>
       </c>
-      <c r="CH4" s="2">
+      <c r="Q4" s="2">
         <v>37</v>
       </c>
-      <c r="CI4" s="2">
+      <c r="R4" s="2">
         <v>67</v>
       </c>
-      <c r="CJ4" s="2">
+      <c r="S4" s="2">
         <v>67</v>
       </c>
-      <c r="CK4" s="2">
+      <c r="T4" s="2">
         <v>61</v>
       </c>
-      <c r="CL4" s="2">
+      <c r="U4" s="2">
         <v>58</v>
       </c>
-      <c r="CM4" s="2">
+      <c r="V4" s="2">
         <v>91</v>
       </c>
-      <c r="CN4" s="2">
+      <c r="W4" s="2">
         <v>77</v>
       </c>
-      <c r="CO4" s="2">
+      <c r="X4" s="2">
         <v>57</v>
       </c>
-      <c r="CP4" s="2">
+      <c r="Y4" s="2">
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="70:94">
-      <c r="BR5" t="s">
+    <row r="5" spans="1:25">
+      <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="BS5" s="2">
+      <c r="B5" s="2">
         <v>36</v>
       </c>
-      <c r="BT5" s="2">
+      <c r="C5" s="2">
         <v>-23</v>
       </c>
-      <c r="BU5" s="2">
+      <c r="D5" s="2">
         <v>56</v>
       </c>
-      <c r="BV5" s="2">
+      <c r="E5" s="2">
         <v>73</v>
       </c>
-      <c r="BW5" s="2">
+      <c r="F5" s="2">
         <v>64</v>
       </c>
-      <c r="BX5" s="2">
+      <c r="G5" s="2">
         <v>34</v>
       </c>
-      <c r="BY5" s="2">
+      <c r="H5" s="2">
         <v>67</v>
       </c>
-      <c r="BZ5" s="2">
+      <c r="I5" s="2">
         <v>71</v>
       </c>
-      <c r="CA5" s="2">
+      <c r="J5" s="2">
         <v>61</v>
       </c>
-      <c r="CB5" s="2">
+      <c r="K5" s="2">
         <v>57</v>
       </c>
-      <c r="CC5" s="2">
+      <c r="L5" s="2">
         <v>67</v>
       </c>
-      <c r="CD5" s="2">
+      <c r="M5" s="2">
         <v>41</v>
       </c>
-      <c r="CE5" s="2">
+      <c r="N5" s="2">
         <v>70</v>
       </c>
-      <c r="CF5" s="2">
+      <c r="O5" s="2">
         <v>39</v>
       </c>
-      <c r="CG5" s="2">
+      <c r="P5" s="2">
         <v>-4</v>
       </c>
-      <c r="CH5" s="2">
+      <c r="Q5" s="2">
         <v>67</v>
       </c>
-      <c r="CI5" s="2">
+      <c r="R5" s="2">
         <v>28</v>
       </c>
-      <c r="CJ5" s="2">
+      <c r="S5" s="2">
         <v>48</v>
       </c>
-      <c r="CK5" s="2">
+      <c r="T5" s="2">
         <v>85</v>
       </c>
-      <c r="CL5" s="2">
+      <c r="U5" s="2">
         <v>58</v>
       </c>
-      <c r="CM5" s="2">
+      <c r="V5" s="2">
         <v>-3</v>
       </c>
-      <c r="CN5" s="2">
+      <c r="W5" s="2">
         <v>48</v>
       </c>
-      <c r="CO5" s="2">
+      <c r="X5" s="2">
         <v>22</v>
       </c>
-      <c r="CP5" s="2">
+      <c r="Y5" s="2">
         <v>83</v>
       </c>
     </row>
-    <row r="6" spans="70:94">
-      <c r="BR6" t="s">
+    <row r="6" spans="1:25">
+      <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="BS6" s="2">
+      <c r="B6" s="2">
         <v>10</v>
       </c>
-      <c r="BT6" s="2">
+      <c r="C6" s="2">
         <v>26</v>
       </c>
-      <c r="BU6" s="2">
+      <c r="D6" s="2">
         <v>19</v>
       </c>
-      <c r="BV6" s="2">
+      <c r="E6" s="2">
         <v>13</v>
       </c>
-      <c r="BW6" s="2">
+      <c r="F6" s="2">
         <v>27</v>
       </c>
-      <c r="BX6" s="2">
+      <c r="G6" s="2">
         <v>31</v>
       </c>
-      <c r="BY6" s="2">
+      <c r="H6" s="2">
         <v>42</v>
       </c>
-      <c r="BZ6" s="2">
+      <c r="I6" s="2">
         <v>16</v>
       </c>
-      <c r="CA6" s="2">
+      <c r="J6" s="2">
         <v>-8</v>
       </c>
-      <c r="CB6" s="2">
+      <c r="K6" s="2">
         <v>4</v>
       </c>
-      <c r="CC6" s="2">
+      <c r="L6" s="2">
         <v>-36</v>
       </c>
-      <c r="CD6" s="2">
+      <c r="M6" s="2">
         <v>16</v>
       </c>
-      <c r="CE6" s="2">
+      <c r="N6" s="2">
         <v>27</v>
       </c>
-      <c r="CF6" s="2">
+      <c r="O6" s="2">
         <v>24</v>
       </c>
-      <c r="CG6" s="2">
+      <c r="P6" s="2">
         <v>35</v>
       </c>
-      <c r="CH6" s="2">
+      <c r="Q6" s="2">
         <v>23</v>
       </c>
-      <c r="CI6" s="2">
+      <c r="R6" s="2">
         <v>46</v>
       </c>
-      <c r="CJ6" s="2">
+      <c r="S6" s="2">
         <v>5</v>
       </c>
-      <c r="CK6" s="2">
+      <c r="T6" s="2">
         <v>27</v>
       </c>
-      <c r="CL6" s="2">
+      <c r="U6" s="2">
         <v>29</v>
       </c>
-      <c r="CM6" s="2">
+      <c r="V6" s="2">
         <v>42</v>
       </c>
-      <c r="CN6" s="2">
+      <c r="W6" s="2">
         <v>9</v>
       </c>
-      <c r="CO6" s="2">
+      <c r="X6" s="2">
         <v>39</v>
       </c>
-      <c r="CP6" s="2">
+      <c r="Y6" s="2">
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="70:94">
-      <c r="BR7" t="s">
+    <row r="7" spans="1:25">
+      <c r="A7" t="s">
         <v>9</v>
       </c>
-      <c r="BS7" s="2">
+      <c r="B7" s="2">
         <v>14</v>
       </c>
-      <c r="BT7" s="2">
+      <c r="C7" s="2">
         <v>47</v>
       </c>
-      <c r="BU7" s="2">
+      <c r="D7" s="2">
         <v>10</v>
       </c>
-      <c r="BV7" s="2">
+      <c r="E7" s="2">
         <v>40</v>
       </c>
-      <c r="BW7" s="2">
+      <c r="F7" s="2">
         <v>12</v>
       </c>
-      <c r="BX7" s="2">
+      <c r="G7" s="2">
         <v>8</v>
       </c>
-      <c r="BY7" s="2">
+      <c r="H7" s="2">
         <v>-13</v>
       </c>
-      <c r="BZ7" s="2">
+      <c r="I7" s="2">
         <v>25</v>
       </c>
-      <c r="CA7" s="2">
+      <c r="J7" s="2">
         <v>6</v>
       </c>
-      <c r="CB7" s="2">
+      <c r="K7" s="2">
         <v>22</v>
       </c>
-      <c r="CC7" s="2">
+      <c r="L7" s="2">
         <v>37</v>
       </c>
-      <c r="CD7" s="2">
+      <c r="M7" s="2">
         <v>25</v>
       </c>
-      <c r="CE7" s="2">
+      <c r="N7" s="2">
         <v>15</v>
       </c>
-      <c r="CF7" s="2">
+      <c r="O7" s="2">
         <v>-9</v>
       </c>
-      <c r="CG7" s="2">
+      <c r="P7" s="2">
         <v>43</v>
       </c>
-      <c r="CH7" s="2">
+      <c r="Q7" s="2">
         <v>7</v>
       </c>
-      <c r="CI7" s="2">
+      <c r="R7" s="2">
         <v>13</v>
       </c>
-      <c r="CJ7" s="2">
+      <c r="S7" s="2">
         <v>15</v>
       </c>
-      <c r="CK7" s="2">
+      <c r="T7" s="2">
         <v>13</v>
       </c>
-      <c r="CL7" s="2">
+      <c r="U7" s="2">
         <v>45</v>
       </c>
-      <c r="CM7" s="2">
+      <c r="V7" s="2">
         <v>54</v>
       </c>
-      <c r="CN7" s="2">
+      <c r="W7" s="2">
         <v>24</v>
       </c>
-      <c r="CO7" s="2">
+      <c r="X7" s="2">
         <v>-5</v>
       </c>
-      <c r="CP7" s="2">
+      <c r="Y7" s="2">
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="70:94">
-      <c r="BR8" t="s">
+    <row r="8" spans="1:25">
+      <c r="A8" t="s">
         <v>13</v>
       </c>
-      <c r="BS8" s="2">
+      <c r="B8" s="2">
         <v>-10</v>
       </c>
-      <c r="BT8" s="2">
+      <c r="C8" s="2">
         <v>42</v>
       </c>
-      <c r="BU8" s="2">
+      <c r="D8" s="2">
         <v>14</v>
       </c>
-      <c r="BV8" s="2">
+      <c r="E8" s="2">
         <v>22</v>
       </c>
-      <c r="BW8" s="2">
+      <c r="F8" s="2">
         <v>18</v>
       </c>
-      <c r="BX8" s="2">
+      <c r="G8" s="2">
         <v>-6</v>
       </c>
-      <c r="BY8" s="2">
+      <c r="H8" s="2">
         <v>24</v>
       </c>
-      <c r="BZ8" s="2">
+      <c r="I8" s="2">
         <v>31</v>
       </c>
-      <c r="CA8" s="2">
+      <c r="J8" s="2">
         <v>35</v>
       </c>
-      <c r="CB8" s="2">
+      <c r="K8" s="2">
         <v>-4</v>
       </c>
-      <c r="CC8" s="2">
+      <c r="L8" s="2">
         <v>34</v>
       </c>
-      <c r="CD8" s="2">
+      <c r="M8" s="2">
         <v>-35</v>
       </c>
-      <c r="CE8" s="2">
+      <c r="N8" s="2">
         <v>17</v>
       </c>
-      <c r="CF8" s="2">
+      <c r="O8" s="2">
         <v>29</v>
       </c>
-      <c r="CG8" s="2">
+      <c r="P8" s="2">
         <v>38</v>
       </c>
-      <c r="CH8" s="2">
+      <c r="Q8" s="2">
         <v>27</v>
       </c>
-      <c r="CI8" s="2">
+      <c r="R8" s="2">
         <v>41</v>
       </c>
-      <c r="CJ8" s="2">
+      <c r="S8" s="2">
         <v>16</v>
       </c>
-      <c r="CK8" s="2">
+      <c r="T8" s="2">
         <v>34</v>
       </c>
-      <c r="CL8" s="2">
+      <c r="U8" s="2">
         <v>-10</v>
       </c>
-      <c r="CM8" s="2">
+      <c r="V8" s="2">
         <v>47</v>
       </c>
-      <c r="CN8" s="2">
+      <c r="W8" s="2">
         <v>30</v>
       </c>
-      <c r="CO8" s="2">
+      <c r="X8" s="2">
         <v>22</v>
       </c>
-      <c r="CP8" s="2">
+      <c r="Y8" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="70:94">
-      <c r="BR9" t="s">
+    <row r="9" spans="1:25">
+      <c r="A9" t="s">
         <v>1</v>
       </c>
-      <c r="BS9" s="2">
+      <c r="B9" s="2">
         <v>1</v>
       </c>
-      <c r="BT9" s="2">
+      <c r="C9" s="2">
         <v>4</v>
       </c>
-      <c r="BU9" s="2">
+      <c r="D9" s="2">
         <v>9</v>
       </c>
-      <c r="BV9" s="2">
+      <c r="E9" s="2">
         <v>18</v>
       </c>
-      <c r="BW9" s="2">
+      <c r="F9" s="2">
         <v>11</v>
       </c>
-      <c r="BX9" s="2">
+      <c r="G9" s="2">
         <v>13</v>
       </c>
-      <c r="BY9" s="2">
+      <c r="H9" s="2">
         <v>14</v>
       </c>
-      <c r="BZ9" s="2">
+      <c r="I9" s="2">
         <v>-4</v>
       </c>
-      <c r="CA9" s="2">
+      <c r="J9" s="2">
         <v>1</v>
       </c>
-      <c r="CB9" s="2">
+      <c r="K9" s="2">
         <v>31</v>
       </c>
-      <c r="CC9" s="2">
+      <c r="L9" s="2">
         <v>24</v>
       </c>
-      <c r="CD9" s="2">
+      <c r="M9" s="2">
         <v>33</v>
       </c>
-      <c r="CE9" s="2">
+      <c r="N9" s="2">
         <v>20</v>
       </c>
-      <c r="CF9" s="2">
+      <c r="O9" s="2">
         <v>45</v>
       </c>
-      <c r="CG9" s="2">
+      <c r="P9" s="2">
         <v>41</v>
       </c>
-      <c r="CH9" s="2">
+      <c r="Q9" s="2">
         <v>-11</v>
       </c>
-      <c r="CI9" s="2">
+      <c r="R9" s="2">
         <v>-2</v>
       </c>
-      <c r="CJ9" s="2">
+      <c r="S9" s="2">
         <v>37</v>
       </c>
-      <c r="CK9" s="2">
+      <c r="T9" s="2">
         <v>-12</v>
       </c>
-      <c r="CL9" s="2">
+      <c r="U9" s="2">
         <v>2</v>
       </c>
-      <c r="CM9" s="2">
+      <c r="V9" s="2">
         <v>9</v>
       </c>
-      <c r="CN9" s="2">
+      <c r="W9" s="2">
         <v>-8</v>
       </c>
-      <c r="CO9" s="2">
+      <c r="X9" s="2">
         <v>21</v>
       </c>
-      <c r="CP9" s="2">
+      <c r="Y9" s="2">
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="70:94">
-      <c r="BR10" t="s">
+    <row r="10" spans="1:25">
+      <c r="A10" t="s">
         <v>11</v>
       </c>
-      <c r="BS10" s="2">
+      <c r="B10" s="2">
         <v>3</v>
       </c>
-      <c r="BT10" s="2">
+      <c r="C10" s="2">
         <v>12</v>
       </c>
-      <c r="BU10" s="2">
+      <c r="D10" s="2">
         <v>0</v>
       </c>
-      <c r="BV10" s="2">
+      <c r="E10" s="2">
         <v>-22</v>
       </c>
-      <c r="BW10" s="2">
+      <c r="F10" s="2">
         <v>10</v>
       </c>
-      <c r="BX10" s="2">
+      <c r="G10" s="2">
         <v>9</v>
       </c>
-      <c r="BY10" s="2">
+      <c r="H10" s="2">
         <v>13</v>
       </c>
-      <c r="BZ10" s="2">
+      <c r="I10" s="2">
         <v>7</v>
       </c>
-      <c r="CA10" s="2">
+      <c r="J10" s="2">
         <v>52</v>
       </c>
-      <c r="CB10" s="2">
+      <c r="K10" s="2">
         <v>26</v>
       </c>
-      <c r="CC10" s="2">
+      <c r="L10" s="2">
         <v>45</v>
       </c>
-      <c r="CD10" s="2">
+      <c r="M10" s="2">
         <v>14</v>
       </c>
-      <c r="CE10" s="2">
+      <c r="N10" s="2">
         <v>24</v>
       </c>
-      <c r="CF10" s="2">
+      <c r="O10" s="2">
         <v>35</v>
       </c>
-      <c r="CG10" s="2">
+      <c r="P10" s="2">
         <v>14</v>
       </c>
-      <c r="CH10" s="2">
+      <c r="Q10" s="2">
         <v>-2</v>
       </c>
-      <c r="CI10" s="2">
+      <c r="R10" s="2">
         <v>17</v>
       </c>
-      <c r="CJ10" s="2">
+      <c r="S10" s="2">
         <v>-4</v>
       </c>
-      <c r="CK10" s="2">
+      <c r="T10" s="2">
         <v>25</v>
       </c>
-      <c r="CL10" s="2">
+      <c r="U10" s="2">
         <v>2</v>
       </c>
-      <c r="CM10" s="2">
+      <c r="V10" s="2">
         <v>-9</v>
       </c>
-      <c r="CN10" s="2">
+      <c r="W10" s="2">
         <v>-8</v>
       </c>
-      <c r="CO10" s="2">
+      <c r="X10" s="2">
         <v>4</v>
       </c>
-      <c r="CP10" s="2">
+      <c r="Y10" s="2">
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="70:94">
-      <c r="BR11" t="s">
+    <row r="11" spans="1:25">
+      <c r="A11" t="s">
         <v>5</v>
       </c>
-      <c r="BS11" s="2">
+      <c r="B11" s="2">
         <v>-14</v>
       </c>
-      <c r="BT11" s="2">
+      <c r="C11" s="2">
         <v>-6</v>
       </c>
-      <c r="BU11" s="2">
+      <c r="D11" s="2">
         <v>9</v>
       </c>
-      <c r="BV11" s="2">
+      <c r="E11" s="2">
         <v>22</v>
       </c>
-      <c r="BW11" s="2">
+      <c r="F11" s="2">
         <v>-6</v>
       </c>
-      <c r="BX11" s="2">
+      <c r="G11" s="2">
         <v>10</v>
       </c>
-      <c r="BY11" s="2">
+      <c r="H11" s="2">
         <v>10</v>
       </c>
-      <c r="BZ11" s="2">
+      <c r="I11" s="2">
         <v>-11</v>
       </c>
-      <c r="CA11" s="2">
+      <c r="J11" s="2">
         <v>31</v>
       </c>
-      <c r="CB11" s="2">
+      <c r="K11" s="2">
         <v>11</v>
       </c>
-      <c r="CC11" s="2">
+      <c r="L11" s="2">
         <v>17</v>
       </c>
-      <c r="CD11" s="2">
+      <c r="M11" s="2">
         <v>5</v>
       </c>
-      <c r="CE11" s="2">
+      <c r="N11" s="2">
         <v>-13</v>
       </c>
-      <c r="CF11" s="2">
+      <c r="O11" s="2">
         <v>2</v>
       </c>
-      <c r="CG11" s="2">
+      <c r="P11" s="2">
         <v>14</v>
       </c>
-      <c r="CH11" s="2">
+      <c r="Q11" s="2">
         <v>6</v>
       </c>
-      <c r="CI11" s="2">
+      <c r="R11" s="2">
         <v>7</v>
       </c>
-      <c r="CJ11" s="2">
+      <c r="S11" s="2">
         <v>6</v>
       </c>
-      <c r="CK11" s="2">
+      <c r="T11" s="2">
         <v>18</v>
       </c>
-      <c r="CL11" s="2">
+      <c r="U11" s="2">
         <v>14</v>
       </c>
-      <c r="CM11" s="2">
+      <c r="V11" s="2">
         <v>12</v>
       </c>
-      <c r="CN11" s="2">
+      <c r="W11" s="2">
         <v>3</v>
       </c>
-      <c r="CO11" s="2">
+      <c r="X11" s="2">
         <v>14</v>
       </c>
-      <c r="CP11" s="2">
+      <c r="Y11" s="2">
         <v>4</v>
       </c>
     </row>
@@ -15493,13 +15529,13 @@
   <sheetPr>
     <tabColor theme="5"/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="B1">
         <v>1</v>
       </c>
@@ -15509,8 +15545,11 @@
       <c r="D1">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -15523,8 +15562,11 @@
       <c r="D2">
         <v>92</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="E2">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -15537,8 +15579,11 @@
       <c r="D3">
         <v>72</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="E3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -15551,8 +15596,11 @@
       <c r="D4">
         <v>25</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="E4">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -15565,8 +15613,11 @@
       <c r="D5">
         <v>75</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="E5">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -15579,8 +15630,11 @@
       <c r="D6">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="1:4">
+      <c r="E6">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -15593,8 +15647,11 @@
       <c r="D7">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="1:4">
+      <c r="E7">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -15607,8 +15664,11 @@
       <c r="D8">
         <v>-12</v>
       </c>
-    </row>
-    <row r="9" spans="1:4">
+      <c r="E8">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -15621,8 +15681,11 @@
       <c r="D9">
         <v>-4</v>
       </c>
-    </row>
-    <row r="10" spans="1:4">
+      <c r="E9">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -15635,8 +15698,11 @@
       <c r="D10">
         <v>23</v>
       </c>
-    </row>
-    <row r="11" spans="1:4">
+      <c r="E10">
+        <v>-27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11" t="s">
         <v>13</v>
       </c>
@@ -15649,8 +15715,11 @@
       <c r="D11">
         <v>18</v>
       </c>
-    </row>
-    <row r="12" spans="1:4">
+      <c r="E11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -15662,6 +15731,9 @@
       </c>
       <c r="D12">
         <v>5</v>
+      </c>
+      <c r="E12">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cont. wiring up the optimizer
</commit_message>
<xml_diff>
--- a/data/raw/newHistPointAndPrice.xlsx
+++ b/data/raw/newHistPointAndPrice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E3D94F4-1DE9-4EAA-B3B4-0BEA363766A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95FA67B4-8435-4B01-8737-879E137EAA90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" firstSheet="7" activeTab="17" xr2:uid="{2D04FC15-E09F-4251-B381-E10D89E9EC62}"/>
+    <workbookView xWindow="-21697" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="864" firstSheet="10" activeTab="16" xr2:uid="{2D04FC15-E09F-4251-B381-E10D89E9EC62}"/>
   </bookViews>
   <sheets>
     <sheet name="2023ConstructorPrice" sheetId="1" r:id="rId1"/>
@@ -10799,6 +10799,9 @@
   </sheetPr>
   <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="11" max="11" width="12.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
adding race_id column to budget and team config
</commit_message>
<xml_diff>
--- a/data/raw/newHistPointAndPrice.xlsx
+++ b/data/raw/newHistPointAndPrice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jackg\code\F1Fantasy\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71DFD566-76F8-485C-9648-6FD827505BCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62438A3D-2263-46AB-8609-31523894EAD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="864" firstSheet="1" activeTab="3" xr2:uid="{2D04FC15-E09F-4251-B381-E10D89E9EC62}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="864" firstSheet="10" activeTab="16" xr2:uid="{2D04FC15-E09F-4251-B381-E10D89E9EC62}"/>
   </bookViews>
   <sheets>
     <sheet name="2023ConstructorPrice" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="89">
   <si>
     <t>Red Bull Racing</t>
   </si>
@@ -320,6 +320,9 @@
   </si>
   <si>
     <t>PER</t>
+  </si>
+  <si>
+    <t>race_id</t>
   </si>
 </sst>
 </file>
@@ -10944,427 +10947,460 @@
   <sheetPr>
     <tabColor theme="5" tint="0.39997558519241921"/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="11" max="11" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" t="s">
         <v>44</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>47</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>48</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>49</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>50</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>51</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>52</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>53</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>54</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
-      <c r="A2" t="s">
+    <row r="2" spans="1:13">
+      <c r="A2">
+        <v>73</v>
+      </c>
+      <c r="B2" t="s">
         <v>56</v>
       </c>
-      <c r="B2">
+      <c r="C2">
         <v>2026</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>57</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>58</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>59</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>60</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>61</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>62</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>58</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
-      <c r="A3" t="s">
+    <row r="3" spans="1:13">
+      <c r="A3">
+        <v>73</v>
+      </c>
+      <c r="B3" t="s">
         <v>64</v>
       </c>
-      <c r="B3">
+      <c r="C3">
         <v>2026</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>1</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>65</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>10</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>58</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>66</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>60</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>61</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>62</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>58</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="4" spans="1:12">
-      <c r="A4" t="s">
+    <row r="4" spans="1:13">
+      <c r="A4">
+        <v>74</v>
+      </c>
+      <c r="B4" t="s">
         <v>68</v>
       </c>
-      <c r="B4">
+      <c r="C4">
         <v>2026</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>2</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>69</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>10</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>58</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>70</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>60</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>61</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>62</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>58</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:12">
-      <c r="A5" t="s">
+    <row r="5" spans="1:13">
+      <c r="A5">
+        <v>74</v>
+      </c>
+      <c r="B5" t="s">
         <v>71</v>
       </c>
-      <c r="B5">
+      <c r="C5">
         <v>2026</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>2</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>69</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>10</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>58</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>70</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>72</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>73</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>74</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>58</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:12">
-      <c r="A6" t="s">
+    <row r="6" spans="1:13">
+      <c r="A6">
         <v>75</v>
       </c>
-      <c r="B6">
+      <c r="B6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C6">
         <v>2026</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>3</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>69</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>10</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>76</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>70</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>66</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>60</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>62</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>76</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="1:12">
-      <c r="A7" t="s">
+    <row r="7" spans="1:13">
+      <c r="A7">
+        <v>75</v>
+      </c>
+      <c r="B7" t="s">
         <v>77</v>
       </c>
-      <c r="B7">
+      <c r="C7">
         <v>2026</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>3</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>69</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>10</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>78</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>70</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>72</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>73</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>74</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>78</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="1:12">
-      <c r="A8" t="s">
+    <row r="8" spans="1:13">
+      <c r="A8">
+        <v>76</v>
+      </c>
+      <c r="B8" t="s">
         <v>80</v>
       </c>
-      <c r="B8">
+      <c r="C8">
         <v>2026</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <v>6</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>69</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>10</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>76</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>70</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>66</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>81</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>62</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>76</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:12">
-      <c r="A9" t="s">
+    <row r="9" spans="1:13">
+      <c r="A9">
+        <v>76</v>
+      </c>
+      <c r="B9" t="s">
         <v>82</v>
       </c>
-      <c r="B9">
+      <c r="C9">
         <v>2026</v>
       </c>
-      <c r="C9">
+      <c r="D9">
         <v>6</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>69</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>10</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>83</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>70</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>72</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>74</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>60</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>83</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="10" spans="1:12">
-      <c r="A10" t="s">
+    <row r="10" spans="1:13">
+      <c r="A10">
+        <v>77</v>
+      </c>
+      <c r="B10" t="s">
         <v>80</v>
       </c>
-      <c r="B10">
+      <c r="C10">
         <v>2026</v>
       </c>
-      <c r="C10">
+      <c r="D10">
         <v>7</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>69</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>57</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>76</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>73</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>60</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>81</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>85</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>76</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:12">
-      <c r="A11" t="s">
+    <row r="11" spans="1:13">
+      <c r="A11">
+        <v>77</v>
+      </c>
+      <c r="B11" t="s">
         <v>82</v>
       </c>
-      <c r="B11">
+      <c r="C11">
         <v>2026</v>
       </c>
-      <c r="C11">
+      <c r="D11">
         <v>7</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>69</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>10</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>86</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>62</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>74</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>87</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>70</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>86</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>67</v>
       </c>
     </row>
@@ -11378,83 +11414,104 @@
   <sheetPr>
     <tabColor theme="5" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" t="s">
         <v>45</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>46</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:4">
       <c r="A2">
+        <v>73</v>
+      </c>
+      <c r="B2">
         <v>2026</v>
       </c>
-      <c r="B2">
+      <c r="C2">
         <v>1</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:4">
       <c r="A3">
+        <v>74</v>
+      </c>
+      <c r="B3">
         <v>2026</v>
       </c>
-      <c r="B3">
+      <c r="C3">
         <v>2</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>100.9</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:4">
       <c r="A4">
+        <v>75</v>
+      </c>
+      <c r="B4">
         <v>2026</v>
       </c>
-      <c r="B4">
+      <c r="C4">
         <v>3</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>103.1</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:4">
       <c r="A5">
+        <v>76</v>
+      </c>
+      <c r="B5">
         <v>2026</v>
       </c>
-      <c r="B5">
+      <c r="C5">
         <v>6</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>104.2</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:4">
       <c r="A6">
+        <v>77</v>
+      </c>
+      <c r="B6">
         <v>2026</v>
       </c>
-      <c r="B6">
+      <c r="C6">
         <v>7</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>105.1</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:4">
       <c r="A7">
+        <v>78</v>
+      </c>
+      <c r="B7">
         <v>2026</v>
       </c>
-      <c r="B7">
+      <c r="C7">
         <v>8</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>105.6</v>
       </c>
     </row>

</xml_diff>